<commit_message>
Update settings to include Notion integration commands
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I73"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2327,16 +2327,219 @@
         <v>Naukri quick-apply (auto)</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
+        <v>13/5/2026, 4:22:14 pm</v>
+      </c>
+      <c r="C67" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Orcapod Consulting Services Private Limited</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Hyderabad, Mumbai, Bengaluru</v>
+      </c>
+      <c r="G67" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-orcapod-consulting-services-mumbai-hyderabad-bengaluru-6-to-9-years-120526012609</v>
+      </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
+      <c r="I67" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
+        <v>13/5/2026, 4:23:20 pm</v>
+      </c>
+      <c r="C68" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Java Full Stack Developer : Hyderabad</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Oracle</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G68" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-hyderabad-oracle-hyderabad-4-to-6-years-130126035194</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
+        <v>13/5/2026, 4:23:27 pm</v>
+      </c>
+      <c r="C69" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Java Full Stack Developer @ Pan India</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Hyderabad, Bengaluru, Delhi / NCR</v>
+      </c>
+      <c r="G69" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-pan-india-infosys-hyderabad-bengaluru-delhi-ncr-5-to-8-years-270426033372</v>
+      </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+      <c r="I69" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
+        <v>13/5/2026, 4:24:22 pm</v>
+      </c>
+      <c r="C70" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Spruce Infotech</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G70" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-spruce-infotech-hyderabad-6-to-10-years-120526008969</v>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
+        <v>13/5/2026, 4:24:55 pm</v>
+      </c>
+      <c r="C71" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Mern Full Stack Developer</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G71" t="str">
+        <v>https://www.naukri.com/job-listings-mern-full-stack-developer-tata-consultancy-services-hyderabad-pune-bengaluru-5-to-10-years-280426018648</v>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+      <c r="I71" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
+        <v>13/5/2026, 4:25:10 pm</v>
+      </c>
+      <c r="C72" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D72" t="str">
+        <v>iOS Developer</v>
+      </c>
+      <c r="E72" t="str">
+        <v>E-Ring</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Hyderabad(Madhapur)</v>
+      </c>
+      <c r="G72" t="str">
+        <v>https://www.naukri.com/job-listings-ios-developer-e-ring-it-solutions-pvt-ltd-hyderabad-3-to-5-years-160426026742</v>
+      </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
+        <v>13/5/2026, 4:35:21 pm</v>
+      </c>
+      <c r="C73" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Orcapod Consulting Services Private Limited</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Hyderabad, Mumbai, Bengaluru</v>
+      </c>
+      <c r="G73" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-orcapod-consulting-services-mumbai-hyderabad-bengaluru-6-to-10-years-120526012609</v>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+      <c r="I73" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I73"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I329"/>
+  <dimension ref="A1:I359"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -11890,9 +12093,879 @@
         <v>External — apply manually</v>
       </c>
     </row>
+    <row r="330">
+      <c r="A330">
+        <v>329</v>
+      </c>
+      <c r="B330" t="str">
+        <v>13/5/2026, 4:21:09 pm</v>
+      </c>
+      <c r="C330" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F330" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G330" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-060526936897</v>
+      </c>
+      <c r="H330" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500973-S2009842_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I330" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331">
+        <v>330</v>
+      </c>
+      <c r="B331" t="str">
+        <v>13/5/2026, 4:21:15 pm</v>
+      </c>
+      <c r="C331" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Full Stack Engineer</v>
+      </c>
+      <c r="E331" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F331" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G331" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526917631</v>
+      </c>
+      <c r="H331" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5272773-S1947288_en&amp;title=Full+Stack+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I331" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332">
+        <v>331</v>
+      </c>
+      <c r="B332" t="str">
+        <v>13/5/2026, 4:21:21 pm</v>
+      </c>
+      <c r="C332" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D332" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E332" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F332" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G332" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-110526917482</v>
+      </c>
+      <c r="H332" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5069755-S1878279_en&amp;title=Software+Development+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I332" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333">
+        <v>332</v>
+      </c>
+      <c r="B333" t="str">
+        <v>13/5/2026, 4:21:27 pm</v>
+      </c>
+      <c r="C333" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G333" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526928187</v>
+      </c>
+      <c r="H333" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5307482-S1938182_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I333" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334">
+        <v>333</v>
+      </c>
+      <c r="B334" t="str">
+        <v>13/5/2026, 4:21:34 pm</v>
+      </c>
+      <c r="C334" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G334" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-050526940199</v>
+      </c>
+      <c r="H334" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5263241-S1945727_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I334" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335">
+        <v>334</v>
+      </c>
+      <c r="B335" t="str">
+        <v>13/5/2026, 4:21:40 pm</v>
+      </c>
+      <c r="C335" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E335" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F335" t="str">
+        <v>Hyderabad, Mumbai</v>
+      </c>
+      <c r="G335" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-2-to-5-years-270426911919</v>
+      </c>
+      <c r="H335" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-R1-S1904898_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I335" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336">
+        <v>335</v>
+      </c>
+      <c r="B336" t="str">
+        <v>13/5/2026, 4:21:47 pm</v>
+      </c>
+      <c r="C336" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F336" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G336" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526918834</v>
+      </c>
+      <c r="H336" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5181452-S1911507_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I336" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337">
+        <v>336</v>
+      </c>
+      <c r="B337" t="str">
+        <v>13/5/2026, 4:21:51 pm</v>
+      </c>
+      <c r="C337" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F337" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G337" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-110526918602</v>
+      </c>
+      <c r="H337" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-R1-S1871732_en&amp;title=Software+Development+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I337" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338">
+        <v>337</v>
+      </c>
+      <c r="B338" t="str">
+        <v>13/5/2026, 4:21:55 pm</v>
+      </c>
+      <c r="C338" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Full Stack Engineer</v>
+      </c>
+      <c r="E338" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F338" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G338" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526917659</v>
+      </c>
+      <c r="H338" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5272776-S1947132_en&amp;title=Full+Stack+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I338" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339">
+        <v>338</v>
+      </c>
+      <c r="B339" t="str">
+        <v>13/5/2026, 4:22:27 pm</v>
+      </c>
+      <c r="C339" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Senior Java Full Stack Developer</v>
+      </c>
+      <c r="E339" t="str">
+        <v>Massmutual Global Business Services India</v>
+      </c>
+      <c r="F339" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G339" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-massmutual-global-business-services-india-llp-hyderabad-10-to-15-years-120526501237</v>
+      </c>
+      <c r="H339" t="str">
+        <v>https://massmutual.wd1.myworkdayjobs.com/en-US/MMINDCareersite/job/Hyderabad-India/Senior-Java-Full-Stack-Developer_R20730</v>
+      </c>
+      <c r="I339" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340">
+        <v>339</v>
+      </c>
+      <c r="B340" t="str">
+        <v>13/5/2026, 4:25:23 pm</v>
+      </c>
+      <c r="C340" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Web Programmer / Full Stack Developer</v>
+      </c>
+      <c r="E340" t="str">
+        <v>Icore Innovations</v>
+      </c>
+      <c r="F340" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G340" t="str">
+        <v>https://www.naukri.com/job-listings-web-programmer-full-stack-developer-icore-innovations-pvt-ltd-hyderabad-1-to-4-years-190126502836</v>
+      </c>
+      <c r="H340" t="str">
+        <v>http://www.icorei.com/main/careers.html</v>
+      </c>
+      <c r="I340" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341">
+        <v>340</v>
+      </c>
+      <c r="B341" t="str">
+        <v>13/5/2026, 4:25:30 pm</v>
+      </c>
+      <c r="C341" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Python Full Stack Developer</v>
+      </c>
+      <c r="E341" t="str">
+        <v>Grid Dynamics</v>
+      </c>
+      <c r="F341" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G341" t="str">
+        <v>https://www.naukri.com/job-listings-python-full-stack-developer-grid-dynamics-hyderabad-3-to-8-years-290126509146</v>
+      </c>
+      <c r="H341" t="str">
+        <v>https://www.griddynamics.com/careers/discover-openings</v>
+      </c>
+      <c r="I341" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342">
+        <v>341</v>
+      </c>
+      <c r="B342" t="str">
+        <v>13/5/2026, 4:25:40 pm</v>
+      </c>
+      <c r="C342" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E342" t="str">
+        <v>Pragma Edge Software Services</v>
+      </c>
+      <c r="F342" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G342" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-pragma-edge-software-services-private-limited-hyderabad-2-to-5-years-290124502269</v>
+      </c>
+      <c r="H342" t="str">
+        <v>https://careers.pragmaedge.com/java-full-stack-developer/</v>
+      </c>
+      <c r="I342" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343">
+        <v>342</v>
+      </c>
+      <c r="B343" t="str">
+        <v>13/5/2026, 4:34:21 pm</v>
+      </c>
+      <c r="C343" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D343" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F343" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G343" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526917478</v>
+      </c>
+      <c r="H343" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5052467-S1874927_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I343" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344">
+        <v>343</v>
+      </c>
+      <c r="B344" t="str">
+        <v>13/5/2026, 4:34:29 pm</v>
+      </c>
+      <c r="C344" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F344" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G344" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526915680</v>
+      </c>
+      <c r="H344" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5230811-S1916683_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I344" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345">
+        <v>344</v>
+      </c>
+      <c r="B345" t="str">
+        <v>13/5/2026, 4:34:44 pm</v>
+      </c>
+      <c r="C345" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D345" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F345" t="str">
+        <v>Hyderabad, Mumbai</v>
+      </c>
+      <c r="G345" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-mumbai-hyderabad-2-to-5-years-040526919557</v>
+      </c>
+      <c r="H345" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5198524-S1908893_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I345" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346">
+        <v>345</v>
+      </c>
+      <c r="B346" t="str">
+        <v>13/5/2026, 4:34:48 pm</v>
+      </c>
+      <c r="C346" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Application Developer</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F346" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G346" t="str">
+        <v>https://www.naukri.com/job-listings-application-developer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526918469</v>
+      </c>
+      <c r="H346" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-4972681-S1855669_en&amp;title=Application+Developer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I346" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347">
+        <v>346</v>
+      </c>
+      <c r="B347" t="str">
+        <v>13/5/2026, 4:34:54 pm</v>
+      </c>
+      <c r="C347" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D347" t="str">
+        <v>Full Stack Engineer</v>
+      </c>
+      <c r="E347" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F347" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G347" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526917885</v>
+      </c>
+      <c r="H347" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5272774-S1947263_en&amp;title=Full+Stack+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I347" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348">
+        <v>347</v>
+      </c>
+      <c r="B348" t="str">
+        <v>13/5/2026, 4:35:00 pm</v>
+      </c>
+      <c r="C348" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F348" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G348" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-160426930759</v>
+      </c>
+      <c r="H348" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500972-S2014297_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I348" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349">
+        <v>348</v>
+      </c>
+      <c r="B349" t="str">
+        <v>13/5/2026, 4:35:09 pm</v>
+      </c>
+      <c r="C349" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F349" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G349" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-160426930508</v>
+      </c>
+      <c r="H349" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500971-S2014336_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I349" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350">
+        <v>349</v>
+      </c>
+      <c r="B350" t="str">
+        <v>13/5/2026, 4:35:13 pm</v>
+      </c>
+      <c r="C350" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E350" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F350" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G350" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-160426929665</v>
+      </c>
+      <c r="H350" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500972-S2014297_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I350" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351">
+        <v>350</v>
+      </c>
+      <c r="B351" t="str">
+        <v>13/5/2026, 4:35:27 pm</v>
+      </c>
+      <c r="C351" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E351" t="str">
+        <v>Upsteer</v>
+      </c>
+      <c r="F351" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G351" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-upsteer-hyderabad-3-to-6-years-270623500218</v>
+      </c>
+      <c r="H351" t="str">
+        <v>https://www.upsteer.com/careers.html</v>
+      </c>
+      <c r="I351" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352">
+        <v>351</v>
+      </c>
+      <c r="B352" t="str">
+        <v>13/5/2026, 4:35:33 pm</v>
+      </c>
+      <c r="C352" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Avontix</v>
+      </c>
+      <c r="F352" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G352" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-avontix-hyderabad-2-to-7-years-250225504341</v>
+      </c>
+      <c r="H352" t="str">
+        <v>https://recruiting.paylocity.com/Recruiting/Jobs/Details/3070946</v>
+      </c>
+      <c r="I352" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353">
+        <v>352</v>
+      </c>
+      <c r="B353" t="str">
+        <v>13/5/2026, 4:35:40 pm</v>
+      </c>
+      <c r="C353" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D353" t="str">
+        <v>Full Stack Developer / Senior Full Stack Developer / Lead FSD</v>
+      </c>
+      <c r="E353" t="str">
+        <v>Tinlas Technologies Private Limited</v>
+      </c>
+      <c r="F353" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G353" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-senior-full-stack-developer-lead-fsd-tinlas-technologies-private-limited-hyderabad-3-to-10-years-201125502125</v>
+      </c>
+      <c r="H353" t="str">
+        <v>https://tinlas.cloud/careers/</v>
+      </c>
+      <c r="I353" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354">
+        <v>353</v>
+      </c>
+      <c r="B354" t="str">
+        <v>13/5/2026, 4:35:46 pm</v>
+      </c>
+      <c r="C354" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Dot Net Full Stack Developer</v>
+      </c>
+      <c r="E354" t="str">
+        <v>Saketh It Solutions</v>
+      </c>
+      <c r="F354" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G354" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-saketh-it-solutions-hyderabad-1-to-2-years-180625500253</v>
+      </c>
+      <c r="H354" t="str">
+        <v>https://www.sakethit.com/jobs/net-full-stack-developer/</v>
+      </c>
+      <c r="I354" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355">
+        <v>354</v>
+      </c>
+      <c r="B355" t="str">
+        <v>13/5/2026, 4:35:52 pm</v>
+      </c>
+      <c r="C355" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Dot Net full stack Developer - Blazor</v>
+      </c>
+      <c r="E355" t="str">
+        <v>GENZEON (INDIA) PRIVATE LIMITED</v>
+      </c>
+      <c r="F355" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G355" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-blazor-genzeon-technology-solutions-private-limited-hyderabad-3-to-7-years-150224501801</v>
+      </c>
+      <c r="H355" t="str">
+        <v>https://www.careers-page.com/genzeon-in/job/L3733W8W</v>
+      </c>
+      <c r="I355" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356">
+        <v>355</v>
+      </c>
+      <c r="B356" t="str">
+        <v>13/5/2026, 4:35:58 pm</v>
+      </c>
+      <c r="C356" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Python Full Stack Developer</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Grid Dynamics</v>
+      </c>
+      <c r="F356" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G356" t="str">
+        <v>https://www.naukri.com/job-listings-python-full-stack-developer-grid-dynamics-hyderabad-3-to-8-years-130126500687</v>
+      </c>
+      <c r="H356" t="str">
+        <v>https://www.griddynamics.com/careers/discover-openings</v>
+      </c>
+      <c r="I356" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357">
+        <v>356</v>
+      </c>
+      <c r="B357" t="str">
+        <v>13/5/2026, 4:36:02 pm</v>
+      </c>
+      <c r="C357" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E357" t="str">
+        <v>Aptsol Global Tech</v>
+      </c>
+      <c r="F357" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G357" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-aptsol-global-tech-pvt-ltd-hyderabad-3-to-5-years-120724501688</v>
+      </c>
+      <c r="H357" t="str">
+        <v>https://www.aptsolglobal.com/careers.php</v>
+      </c>
+      <c r="I357" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358">
+        <v>357</v>
+      </c>
+      <c r="B358" t="str">
+        <v>13/5/2026, 4:36:07 pm</v>
+      </c>
+      <c r="C358" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D358" t="str">
+        <v>MERN Full Stack Developer</v>
+      </c>
+      <c r="E358" t="str">
+        <v>Hiringhood</v>
+      </c>
+      <c r="F358" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G358" t="str">
+        <v>https://www.naukri.com/job-listings-mern-full-stack-developer-hiringhood-hyderabad-3-to-6-years-030624503658</v>
+      </c>
+      <c r="H358" t="str">
+        <v>https://app.pyjamahr.com/careers?company=company&amp;job_id=100261&amp;company_uuid=AF097A8A30</v>
+      </c>
+      <c r="I358" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359">
+        <v>358</v>
+      </c>
+      <c r="B359" t="str">
+        <v>13/5/2026, 4:36:14 pm</v>
+      </c>
+      <c r="C359" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Net Full stack - Developer</v>
+      </c>
+      <c r="E359" t="str">
+        <v>Diensten Tech</v>
+      </c>
+      <c r="F359" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G359" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-diensten-tech-limited-hyderabad-bengaluru-2-to-5-years-030325500357</v>
+      </c>
+      <c r="H359" t="str">
+        <v>https://www.dienstentech.com/jobs/</v>
+      </c>
+      <c r="I359" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I329"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I359"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11950,7 +13023,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I205"/>
+  <dimension ref="A1:I226"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -17908,9 +18981,618 @@
         <v>chatbot_unknown</v>
       </c>
     </row>
+    <row r="206">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="str">
+        <v>13/5/2026, 4:21:01 pm</v>
+      </c>
+      <c r="C206" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Full Stack .NET Developer</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Everi India</v>
+      </c>
+      <c r="F206" t="str">
+        <v>Hyderabad, Chennai</v>
+      </c>
+      <c r="G206" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-net-developer-everi-india-hyderabad-chennai-2-to-5-years-060526025000</v>
+      </c>
+      <c r="H206" t="str">
+        <v/>
+      </c>
+      <c r="I206" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" t="str">
+        <v>13/5/2026, 4:22:07 pm</v>
+      </c>
+      <c r="C207" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D207" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Orcapod Consulting Services Private Limited</v>
+      </c>
+      <c r="F207" t="str">
+        <v>Hybrid - Hyderabad, Mumbai (All Areas), Bengaluru</v>
+      </c>
+      <c r="G207" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-orcapod-consulting-services-hyderabad-bengaluru-mumbai-all-areas-6-to-11-years-130526020790</v>
+      </c>
+      <c r="H207" t="str">
+        <v/>
+      </c>
+      <c r="I207" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" t="str">
+        <v>13/5/2026, 4:22:22 pm</v>
+      </c>
+      <c r="C208" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Python Full stack Developer</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Cognizant</v>
+      </c>
+      <c r="F208" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G208" t="str">
+        <v>https://www.naukri.com/job-listings-python-full-stack-developer-cognizant-hyderabad-6-to-9-years-120526017294</v>
+      </c>
+      <c r="H208" t="str">
+        <v/>
+      </c>
+      <c r="I208" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" t="str">
+        <v>13/5/2026, 4:22:35 pm</v>
+      </c>
+      <c r="C209" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Cerebra</v>
+      </c>
+      <c r="F209" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G209" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-cerebra-hyderabad-6-to-11-years-130526015395</v>
+      </c>
+      <c r="H209" t="str">
+        <v/>
+      </c>
+      <c r="I209" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="str">
+        <v>13/5/2026, 4:22:43 pm</v>
+      </c>
+      <c r="C210" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Happiest Minds Technologies</v>
+      </c>
+      <c r="F210" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G210" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-happiest-minds-technologies-hyderabad-8-to-10-years-130526015244</v>
+      </c>
+      <c r="H210" t="str">
+        <v/>
+      </c>
+      <c r="I210" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="str">
+        <v>13/5/2026, 4:23:10 pm</v>
+      </c>
+      <c r="C211" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Teksystems</v>
+      </c>
+      <c r="F211" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G211" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-teksystems-global-services-hyderabad-bengaluru-5-to-10-years-130226035496</v>
+      </c>
+      <c r="H211" t="str">
+        <v/>
+      </c>
+      <c r="I211" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="str">
+        <v>13/5/2026, 4:23:57 pm</v>
+      </c>
+      <c r="C212" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F212" t="str">
+        <v>Hybrid - Hyderabad, Chennai</v>
+      </c>
+      <c r="G212" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-wipro-hyderabad-chennai-5-to-10-years-130526012872</v>
+      </c>
+      <c r="H212" t="str">
+        <v/>
+      </c>
+      <c r="I212" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="str">
+        <v>13/5/2026, 4:24:04 pm</v>
+      </c>
+      <c r="C213" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Java Full Stack Developer | Java + React |</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F213" t="str">
+        <v>Hybrid - Hyderabad, Pune, Chennai</v>
+      </c>
+      <c r="G213" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-java-react-wipro-hyderabad-pune-chennai-7-to-12-years-120526027177</v>
+      </c>
+      <c r="H213" t="str">
+        <v/>
+      </c>
+      <c r="I213" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="str">
+        <v>13/5/2026, 4:24:12 pm</v>
+      </c>
+      <c r="C214" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Job Opening For Java Full Stack Developer</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Capgemini</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Hybrid - Hyderabad, Pune</v>
+      </c>
+      <c r="G214" t="str">
+        <v>https://www.naukri.com/job-listings-opening-for-java-full-stack-developer-capgemini-hyderabad-pune-5-to-8-years-120526027151</v>
+      </c>
+      <c r="H214" t="str">
+        <v/>
+      </c>
+      <c r="I214" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="str">
+        <v>13/5/2026, 4:24:26 pm</v>
+      </c>
+      <c r="C215" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Walk-in || Java Full Stack Developer</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Hexaware Technologies</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G215" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-hexaware-technologies-hyderabad-chennai-bengaluru-6-to-11-years-111225012381</v>
+      </c>
+      <c r="H215" t="str">
+        <v/>
+      </c>
+      <c r="I215" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="str">
+        <v>13/5/2026, 4:24:30 pm</v>
+      </c>
+      <c r="C216" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Walk-in | Azure Dot Net Full stack Developer</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G216" t="str">
+        <v>https://www.naukri.com/job-listings-walk-in-azure-dot-net-full-stack-developer-tata-consultancy-services-hyderabad-4-to-9-years-100226043886</v>
+      </c>
+      <c r="H216" t="str">
+        <v/>
+      </c>
+      <c r="I216" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="str">
+        <v>13/5/2026, 4:24:33 pm</v>
+      </c>
+      <c r="C217" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Walk-in || Mern Stack Developer</v>
+      </c>
+      <c r="E217" t="str">
+        <v>9X Technology</v>
+      </c>
+      <c r="F217" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G217" t="str">
+        <v>https://www.naukri.com/job-listings-mern-stack-developer-9x-technology-hyderabad-3-to-6-years-130526026100</v>
+      </c>
+      <c r="H217" t="str">
+        <v/>
+      </c>
+      <c r="I217" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="str">
+        <v>13/5/2026, 4:24:37 pm</v>
+      </c>
+      <c r="C218" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D218" t="str">
+        <v>Walk In Drive - Azure + .Net Full Stack Developer</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F218" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G218" t="str">
+        <v>https://www.naukri.com/job-listings-walk-in-drive-azure-net-full-stack-developer-tata-consultancy-services-hyderabad-bengaluru-5-to-10-years-060526017650</v>
+      </c>
+      <c r="H218" t="str">
+        <v/>
+      </c>
+      <c r="I218" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" t="str">
+        <v>13/5/2026, 4:24:45 pm</v>
+      </c>
+      <c r="C219" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D219" t="str">
+        <v>Java (React JS /Node JS)Full Stack Developer -Only 4+yrs</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Tekskills india</v>
+      </c>
+      <c r="F219" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G219" t="str">
+        <v>https://www.naukri.com/job-listings-java-react-js-node-js-full-stack-developer-only-4-yrs-tekskills-hyderabad-4-to-9-years-280426931983</v>
+      </c>
+      <c r="H219" t="str">
+        <v/>
+      </c>
+      <c r="I219" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="str">
+        <v>13/5/2026, 4:25:18 pm</v>
+      </c>
+      <c r="C220" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F220" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G220" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-infosys-hyderabad-3-to-8-years-230426030625</v>
+      </c>
+      <c r="H220" t="str">
+        <v/>
+      </c>
+      <c r="I220" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" t="str">
+        <v>13/5/2026, 4:34:37 pm</v>
+      </c>
+      <c r="C221" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D221" t="str">
+        <v>Node.js Developer</v>
+      </c>
+      <c r="E221" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F221" t="str">
+        <v>Hyderabad, Mumbai, Bengaluru</v>
+      </c>
+      <c r="G221" t="str">
+        <v>https://www.naukri.com/job-listings-node-js-developer-talent-corner-hr-services-pvt-ltd-mumbai-hyderabad-bengaluru-1-to-3-years-280426929733</v>
+      </c>
+      <c r="H221" t="str">
+        <v/>
+      </c>
+      <c r="I221" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" t="str">
+        <v>13/5/2026, 4:36:43 pm</v>
+      </c>
+      <c r="C222" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D222" t="str">
+        <v>Net Full Stack Developer</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F222" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G222" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-infosys-hyderabad-pune-bengaluru-6-to-11-years-270326034575</v>
+      </c>
+      <c r="H222" t="str">
+        <v/>
+      </c>
+      <c r="I222" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223" t="str">
+        <v>13/5/2026, 4:36:51 pm</v>
+      </c>
+      <c r="C223" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D223" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E223" t="str">
+        <v>with one of our Level 5 Client</v>
+      </c>
+      <c r="F223" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G223" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-bcforward-hyderabad-6-to-11-years-230426916125</v>
+      </c>
+      <c r="H223" t="str">
+        <v/>
+      </c>
+      <c r="I223" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224" t="str">
+        <v>13/5/2026, 4:36:59 pm</v>
+      </c>
+      <c r="C224" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D224" t="str">
+        <v>Sr. Java full stack developer</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F224" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G224" t="str">
+        <v>https://www.naukri.com/job-listings-sr-java-full-stack-developer-ideslabs-private-limited-hyderabad-bengaluru-5-to-10-years-220426928702</v>
+      </c>
+      <c r="H224" t="str">
+        <v/>
+      </c>
+      <c r="I224" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225" t="str">
+        <v>13/5/2026, 4:37:06 pm</v>
+      </c>
+      <c r="C225" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D225" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E225" t="str">
+        <v>Staginnovations</v>
+      </c>
+      <c r="F225" t="str">
+        <v>Hyderabad, Chennai, Bengaluru(Karnataka Layout)</v>
+      </c>
+      <c r="G225" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-staginnovations-hyderabad-chennai-bengaluru-5-to-6-years-130426021059</v>
+      </c>
+      <c r="H225" t="str">
+        <v/>
+      </c>
+      <c r="I225" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="str">
+        <v>13/5/2026, 4:37:16 pm</v>
+      </c>
+      <c r="C226" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D226" t="str">
+        <v>Net Full Stack Developer</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F226" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G226" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-infosys-hyderabad-pune-bengaluru-6-to-11-years-100426020328</v>
+      </c>
+      <c r="H226" t="str">
+        <v/>
+      </c>
+      <c r="I226" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I205"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I226"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job application data and enhance Notion integration settings
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I82"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2530,16 +2530,277 @@
         <v>Naukri quick-apply (auto)</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
+        <v>18/5/2026, 2:33:37 pm</v>
+      </c>
+      <c r="C74" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Fullstack sfmc developer with Sql</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Omnicom Global Solutions</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Hybrid - Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G74" t="str">
+        <v>https://www.naukri.com/job-listings-fullstack-sfmc-developer-with-sql-omnicom-global-solutions-hyderabad-bengaluru-1-to-6-years-140526037031</v>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+      <c r="I74" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>18/5/2026, 2:37:09 pm</v>
+      </c>
+      <c r="C75" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Veritis Solutions India Pvt. Ltd.</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Hyderabad/Secunderabad</v>
+      </c>
+      <c r="G75" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-veritis-hyderabad-secunderabad-5-to-10-years-020725029426</v>
+      </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
+      <c r="I75" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>18/5/2026, 2:38:42 pm</v>
+      </c>
+      <c r="C76" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Orcapod Consulting Services Private Limited</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Hyderabad, Mumbai (All Areas), Bengaluru</v>
+      </c>
+      <c r="G76" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-orcapod-consulting-services-hyderabad-bengaluru-mumbai-all-areas-6-to-9-years-150526015136</v>
+      </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
+      <c r="I76" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
+        <v>18/5/2026, 2:38:49 pm</v>
+      </c>
+      <c r="C77" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Orcapod Consulting Services Private Limited</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Hyderabad, Mumbai (All Areas), Bengaluru</v>
+      </c>
+      <c r="G77" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-orcapod-consulting-services-hyderabad-bengaluru-mumbai-all-areas-6-to-9-years-150526013339</v>
+      </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+      <c r="I77" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="str">
+        <v>18/5/2026, 2:39:55 pm</v>
+      </c>
+      <c r="C78" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Full Stack Developer (React &amp; Python) _ Hyderabad @ WFO</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Techouts</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G78" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-react-python-hyderabad-wfo-techouts-hyderabad-4-to-8-years-160526009540</v>
+      </c>
+      <c r="H78" t="str">
+        <v/>
+      </c>
+      <c r="I78" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="str">
+        <v>18/5/2026, 2:40:22 pm</v>
+      </c>
+      <c r="C79" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Job Opportunity Python Full stack Developer-PAN India (Client: TCS)</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Siro Clinpharm</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Hyderabad, Noida, Bengaluru</v>
+      </c>
+      <c r="G79" t="str">
+        <v>https://www.naukri.com/job-listings-opportunity-python-full-stack-developer-pan-india-client-tcs-siro-clinpharm-noida-hyderabad-bengaluru-8-to-13-years-140526013882</v>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="str">
+        <v>18/5/2026, 2:40:37 pm</v>
+      </c>
+      <c r="C80" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Senior .NET Full Stack Developer with Azure</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Cirruslabs</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G80" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-with-azure-cirruslabs-hyderabad-pune-bengaluru-8-to-12-years-090426011270</v>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="str">
+        <v>18/5/2026, 2:42:08 pm</v>
+      </c>
+      <c r="C81" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Hybrid - Hyderabad, Kochi, Chennai</v>
+      </c>
+      <c r="G81" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-wipro-kochi-hyderabad-chennai-5-to-10-years-100725017579</v>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+      <c r="I81" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="str">
+        <v>18/5/2026, 2:42:16 pm</v>
+      </c>
+      <c r="C82" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Hyderabad, Bhubaneswar, Pune</v>
+      </c>
+      <c r="G82" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-bhubaneswar-hyderabad-pune-6-to-10-years-090226017144</v>
+      </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+      <c r="I82" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I82"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I359"/>
+  <dimension ref="A1:I375"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -12963,9 +13224,473 @@
         <v>External — apply manually</v>
       </c>
     </row>
+    <row r="360">
+      <c r="A360">
+        <v>359</v>
+      </c>
+      <c r="B360" t="str">
+        <v>18/5/2026, 2:33:29 pm</v>
+      </c>
+      <c r="C360" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="E360" t="str">
+        <v>Wells Fargo</v>
+      </c>
+      <c r="F360" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G360" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-wells-fargo-international-solutions-private-ltd-hyderabad-2-to-7-years-080526914688</v>
+      </c>
+      <c r="H360" t="str">
+        <v>https://wd1.myworkdaysite.com/en-US/recruiting/wf/WellsFargoJobs/job/Hyderabad-India/Software-Engineer_R-540897</v>
+      </c>
+      <c r="I360" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361">
+        <v>360</v>
+      </c>
+      <c r="B361" t="str">
+        <v>18/5/2026, 2:33:41 pm</v>
+      </c>
+      <c r="C361" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D361" t="str">
+        <v>React Developer</v>
+      </c>
+      <c r="E361" t="str">
+        <v>AIM United Company Ltd</v>
+      </c>
+      <c r="F361" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G361" t="str">
+        <v>https://www.naukri.com/job-listings-react-developer-aim-united-company-ltd-hyderabad-1-to-4-years-150526502479</v>
+      </c>
+      <c r="H361" t="str">
+        <v>https://aim-unitedglobal.com/careers</v>
+      </c>
+      <c r="I361" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362">
+        <v>361</v>
+      </c>
+      <c r="B362" t="str">
+        <v>18/5/2026, 2:33:47 pm</v>
+      </c>
+      <c r="C362" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Full Stack Engineer</v>
+      </c>
+      <c r="E362" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F362" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G362" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-130526939539</v>
+      </c>
+      <c r="H362" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5272778-S1947299_en&amp;title=Full+Stack+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I362" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363">
+        <v>362</v>
+      </c>
+      <c r="B363" t="str">
+        <v>18/5/2026, 2:33:52 pm</v>
+      </c>
+      <c r="C363" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D363" t="str">
+        <v>Node.js Developer</v>
+      </c>
+      <c r="E363" t="str">
+        <v>Vedhas Technology Solutions Llc</v>
+      </c>
+      <c r="F363" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G363" t="str">
+        <v>https://www.naukri.com/job-listings-node-js-developer-vedhas-technology-solutions-llc-hyderabad-2-to-3-years-130526500362</v>
+      </c>
+      <c r="H363" t="str">
+        <v>https://techvedhas.com/hire/</v>
+      </c>
+      <c r="I363" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364">
+        <v>363</v>
+      </c>
+      <c r="B364" t="str">
+        <v>18/5/2026, 2:33:57 pm</v>
+      </c>
+      <c r="C364" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D364" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="E364" t="str">
+        <v>Wells Fargo</v>
+      </c>
+      <c r="F364" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G364" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-wells-fargo-international-solutions-private-ltd-hyderabad-1-to-4-years-110526928370</v>
+      </c>
+      <c r="H364" t="str">
+        <v>https://wd1.myworkdaysite.com/en-US/recruiting/wf/WellsFargoJobs/job/Hyderabad-India/Software-Engineer_R-517308</v>
+      </c>
+      <c r="I364" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365">
+        <v>364</v>
+      </c>
+      <c r="B365" t="str">
+        <v>18/5/2026, 2:34:03 pm</v>
+      </c>
+      <c r="C365" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D365" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E365" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F365" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G365" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526917815</v>
+      </c>
+      <c r="H365" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5395190-S2011446_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I365" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366">
+        <v>365</v>
+      </c>
+      <c r="B366" t="str">
+        <v>18/5/2026, 2:34:07 pm</v>
+      </c>
+      <c r="C366" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F366" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G366" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-150526923821</v>
+      </c>
+      <c r="H366" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobsearch</v>
+      </c>
+      <c r="I366" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367">
+        <v>366</v>
+      </c>
+      <c r="B367" t="str">
+        <v>18/5/2026, 2:34:13 pm</v>
+      </c>
+      <c r="C367" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E367" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F367" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G367" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526918092</v>
+      </c>
+      <c r="H367" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5097342-S1886418_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I367" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368">
+        <v>367</v>
+      </c>
+      <c r="B368" t="str">
+        <v>18/5/2026, 2:34:19 pm</v>
+      </c>
+      <c r="C368" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D368" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E368" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F368" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G368" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-110526916423</v>
+      </c>
+      <c r="H368" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5285850-S1931285_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I368" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369">
+        <v>368</v>
+      </c>
+      <c r="B369" t="str">
+        <v>18/5/2026, 2:34:25 pm</v>
+      </c>
+      <c r="C369" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E369" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F369" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G369" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-040526924888</v>
+      </c>
+      <c r="H369" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-R1-S1888188_en&amp;title=Software+Development+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I369" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370">
+        <v>369</v>
+      </c>
+      <c r="B370" t="str">
+        <v>18/5/2026, 2:34:30 pm</v>
+      </c>
+      <c r="C370" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E370" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F370" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G370" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-040526924039</v>
+      </c>
+      <c r="H370" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5069740-S1878282_en&amp;title=Software+Development+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I370" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371">
+        <v>370</v>
+      </c>
+      <c r="B371" t="str">
+        <v>18/5/2026, 2:37:43 pm</v>
+      </c>
+      <c r="C371" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Jtek Software Solutions</v>
+      </c>
+      <c r="F371" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G371" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-jtek-software-solutions-hyderabad-20-to-30-years-140526503813</v>
+      </c>
+      <c r="H371" t="str">
+        <v>https://jteksoftware.in/jobs/full-stack-developerreact-js-node/</v>
+      </c>
+      <c r="I371" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372">
+        <v>371</v>
+      </c>
+      <c r="B372" t="str">
+        <v>18/5/2026, 2:37:52 pm</v>
+      </c>
+      <c r="C372" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D372" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Ilensys Technologies</v>
+      </c>
+      <c r="F372" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G372" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-ilensys-technologies-hyderabad-5-to-8-years-140526503700</v>
+      </c>
+      <c r="H372" t="str">
+        <v>https://www.ilensys.com/job-details/98</v>
+      </c>
+      <c r="I372" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373">
+        <v>372</v>
+      </c>
+      <c r="B373" t="str">
+        <v>18/5/2026, 2:37:58 pm</v>
+      </c>
+      <c r="C373" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Senior .NET Full Stack Developer</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Devlats</v>
+      </c>
+      <c r="F373" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G373" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-devlats-hyderabad-4-to-9-years-180526503530</v>
+      </c>
+      <c r="H373" t="str">
+        <v>https://careers.devlats.com/job-details/J201</v>
+      </c>
+      <c r="I373" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374">
+        <v>373</v>
+      </c>
+      <c r="B374" t="str">
+        <v>18/5/2026, 2:38:07 pm</v>
+      </c>
+      <c r="C374" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D374" t="str">
+        <v>Senior Java Full Stack Developer</v>
+      </c>
+      <c r="E374" t="str">
+        <v>CGI</v>
+      </c>
+      <c r="F374" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G374" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-cgi-information-systems-and-management-consultants-hyderabad-16-to-17-years-150526503046</v>
+      </c>
+      <c r="H374" t="str">
+        <v>https://cgi.njoyn.com/corp/xweb/xweb.asp?NTKN=c&amp;clid=21001&amp;Page=JobDetails&amp;Jobid=J0426-1700&amp;BRID=1285875&amp;lang=1</v>
+      </c>
+      <c r="I374" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375">
+        <v>374</v>
+      </c>
+      <c r="B375" t="str">
+        <v>18/5/2026, 2:41:33 pm</v>
+      </c>
+      <c r="C375" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D375" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E375" t="str">
+        <v>BTS Infotech</v>
+      </c>
+      <c r="F375" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G375" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-bts-infotech-pvt-ltd-hyderabad-1-to-2-years-111023500264</v>
+      </c>
+      <c r="H375" t="str">
+        <v>https://btsinfotech.com/career.php</v>
+      </c>
+      <c r="I375" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I359"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I375"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -13023,7 +13748,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I226"/>
+  <dimension ref="A1:I253"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -19590,9 +20315,792 @@
         <v>chatbot_unknown</v>
       </c>
     </row>
+    <row r="227">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="str">
+        <v>18/5/2026, 2:33:16 pm</v>
+      </c>
+      <c r="C227" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D227" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Nipum It Solutions Pvt Ltd</v>
+      </c>
+      <c r="F227" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G227" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-spm-hr-solutions-hyderabad-0-to-2-years-140526032036</v>
+      </c>
+      <c r="H227" t="str">
+        <v/>
+      </c>
+      <c r="I227" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228">
+        <v>227</v>
+      </c>
+      <c r="B228" t="str">
+        <v>18/5/2026, 2:33:24 pm</v>
+      </c>
+      <c r="C228" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D228" t="str">
+        <v>Fullstack Developer</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Futuretech Life Care</v>
+      </c>
+      <c r="F228" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G228" t="str">
+        <v>https://www.naukri.com/job-listings-fullstack-developer-futuretech-life-care-hyderabad-2-to-4-years-160526014734</v>
+      </c>
+      <c r="H228" t="str">
+        <v/>
+      </c>
+      <c r="I228" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" t="str">
+        <v>18/5/2026, 2:34:37 pm</v>
+      </c>
+      <c r="C229" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D229" t="str">
+        <v>Job Opportunity For Full Stack Developer</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Virtusa</v>
+      </c>
+      <c r="F229" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G229" t="str">
+        <v>https://www.naukri.com/job-listings-opportunity-for-full-stack-developer-virtusa-hyderabad-4-to-7-years-180526009030</v>
+      </c>
+      <c r="H229" t="str">
+        <v/>
+      </c>
+      <c r="I229" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" t="str">
+        <v>18/5/2026, 2:34:45 pm</v>
+      </c>
+      <c r="C230" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D230" t="str">
+        <v>Azure AI Full Stack Developer</v>
+      </c>
+      <c r="E230" t="str">
+        <v>CMM Level 5 IT Company</v>
+      </c>
+      <c r="F230" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G230" t="str">
+        <v>https://www.naukri.com/job-listings-azure-ai-full-stack-developer-experis-hyderabad-pune-bengaluru-7-to-12-years-150526006907</v>
+      </c>
+      <c r="H230" t="str">
+        <v/>
+      </c>
+      <c r="I230" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" t="str">
+        <v>18/5/2026, 2:34:53 pm</v>
+      </c>
+      <c r="C231" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D231" t="str">
+        <v>Full stack developer</v>
+      </c>
+      <c r="E231" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F231" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G231" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-tekskills-india-private-limited-hyderabad-3-to-8-years-280426930224</v>
+      </c>
+      <c r="H231" t="str">
+        <v/>
+      </c>
+      <c r="I231" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" t="str">
+        <v>18/5/2026, 2:35:01 pm</v>
+      </c>
+      <c r="C232" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D232" t="str">
+        <v>AWS Full Stack Developer (GDC)</v>
+      </c>
+      <c r="E232" t="str">
+        <v>Hitachi Digital Services</v>
+      </c>
+      <c r="F232" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G232" t="str">
+        <v>https://www.naukri.com/job-listings-aws-full-stack-developer-gdc-hitachi-digital-services-hyderabad-pune-bengaluru-8-to-12-years-130526037573</v>
+      </c>
+      <c r="H232" t="str">
+        <v/>
+      </c>
+      <c r="I232" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" t="str">
+        <v>18/5/2026, 2:35:09 pm</v>
+      </c>
+      <c r="C233" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D233" t="str">
+        <v>Full stack Backend Developer</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Apidel Technologies</v>
+      </c>
+      <c r="F233" t="str">
+        <v>Hyderabad, Delhi / NCR</v>
+      </c>
+      <c r="G233" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-backend-developer-apidel-technologies-hyderabad-delhi-ncr-9-to-13-years-130526041284</v>
+      </c>
+      <c r="H233" t="str">
+        <v/>
+      </c>
+      <c r="I233" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" t="str">
+        <v>18/5/2026, 2:35:17 pm</v>
+      </c>
+      <c r="C234" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D234" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E234" t="str">
+        <v>DWPlaceSolutions</v>
+      </c>
+      <c r="F234" t="str">
+        <v>Hyderabad(Madhapur)</v>
+      </c>
+      <c r="G234" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-dwplacesolutions-hyderabad-4-to-6-years-150526027997</v>
+      </c>
+      <c r="H234" t="str">
+        <v/>
+      </c>
+      <c r="I234" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235">
+        <v>234</v>
+      </c>
+      <c r="B235" t="str">
+        <v>18/5/2026, 2:35:44 pm</v>
+      </c>
+      <c r="C235" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D235" t="str">
+        <v>Senior .NET Full Stack Developer</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Independent Recruitment Consultant (freelancer)</v>
+      </c>
+      <c r="F235" t="str">
+        <v>Hyderabad(Nanakramguda)</v>
+      </c>
+      <c r="G235" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-freelancer-hyderabad-4-to-6-years-220426038671</v>
+      </c>
+      <c r="H235" t="str">
+        <v/>
+      </c>
+      <c r="I235" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" t="str">
+        <v>18/5/2026, 2:35:52 pm</v>
+      </c>
+      <c r="C236" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D236" t="str">
+        <v>.NET Full Stack Developer</v>
+      </c>
+      <c r="E236" t="str">
+        <v>S&amp;P Global Market Intelligence</v>
+      </c>
+      <c r="F236" t="str">
+        <v>Hyderabad, Gurugram</v>
+      </c>
+      <c r="G236" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-s-p-capital-iq-india-pvt-ltd-hyderabad-gurugram-3-to-5-years-130526941881</v>
+      </c>
+      <c r="H236" t="str">
+        <v/>
+      </c>
+      <c r="I236" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237">
+        <v>236</v>
+      </c>
+      <c r="B237" t="str">
+        <v>18/5/2026, 2:36:19 pm</v>
+      </c>
+      <c r="C237" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D237" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E237" t="str">
+        <v>IBM</v>
+      </c>
+      <c r="F237" t="str">
+        <v>Hyderabad, Mumbai (All Areas)</v>
+      </c>
+      <c r="G237" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-dynpro-hyderabad-mumbai-all-areas-3-to-7-years-130526038185</v>
+      </c>
+      <c r="H237" t="str">
+        <v/>
+      </c>
+      <c r="I237" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238">
+        <v>237</v>
+      </c>
+      <c r="B238" t="str">
+        <v>18/5/2026, 2:36:47 pm</v>
+      </c>
+      <c r="C238" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D238" t="str">
+        <v>SAP Full Stack Developer (AI Developer)</v>
+      </c>
+      <c r="E238" t="str">
+        <v>CLIENT OF IT SCIENT</v>
+      </c>
+      <c r="F238" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G238" t="str">
+        <v>https://www.naukri.com/job-listings-sap-full-stack-developer-ai-developer-it-scient-hyderabad-pune-bengaluru-6-to-10-years-160526015779</v>
+      </c>
+      <c r="H238" t="str">
+        <v/>
+      </c>
+      <c r="I238" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239">
+        <v>238</v>
+      </c>
+      <c r="B239" t="str">
+        <v>18/5/2026, 2:36:55 pm</v>
+      </c>
+      <c r="C239" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D239" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F239" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G239" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-11-years-180526001042</v>
+      </c>
+      <c r="H239" t="str">
+        <v/>
+      </c>
+      <c r="I239" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240">
+        <v>239</v>
+      </c>
+      <c r="B240" t="str">
+        <v>18/5/2026, 2:37:37 pm</v>
+      </c>
+      <c r="C240" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D240" t="str">
+        <v>SAP Full Stack Developer (AI Developer)</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Tata Consultancy Services(TCS)</v>
+      </c>
+      <c r="F240" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G240" t="str">
+        <v>https://www.naukri.com/job-listings-sap-full-stack-developer-ai-developer-it-scient-hyderabad-chennai-bengaluru-8-to-10-years-150526015391</v>
+      </c>
+      <c r="H240" t="str">
+        <v/>
+      </c>
+      <c r="I240" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241">
+        <v>240</v>
+      </c>
+      <c r="B241" t="str">
+        <v>18/5/2026, 2:38:34 pm</v>
+      </c>
+      <c r="C241" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D241" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E241" t="str">
+        <v>MNC Group</v>
+      </c>
+      <c r="F241" t="str">
+        <v>Hybrid - Hyderabad, Mumbai (All Areas), Pune</v>
+      </c>
+      <c r="G241" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-professional-connect-hyderabad-pune-mumbai-all-areas-6-to-11-years-150526018601</v>
+      </c>
+      <c r="H241" t="str">
+        <v/>
+      </c>
+      <c r="I241" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242">
+        <v>241</v>
+      </c>
+      <c r="B242" t="str">
+        <v>18/5/2026, 2:39:16 pm</v>
+      </c>
+      <c r="C242" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D242" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Quadrant Technologies</v>
+      </c>
+      <c r="F242" t="str">
+        <v>Hybrid - Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G242" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-quadrant-technologies-hyderabad-bengaluru-5-to-10-years-200126040964</v>
+      </c>
+      <c r="H242" t="str">
+        <v/>
+      </c>
+      <c r="I242" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243">
+        <v>242</v>
+      </c>
+      <c r="B243" t="str">
+        <v>18/5/2026, 2:39:43 pm</v>
+      </c>
+      <c r="C243" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D243" t="str">
+        <v>Senior Full Stack Developer (Angular / React &amp; Java)</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Columbus Global</v>
+      </c>
+      <c r="F243" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G243" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-angular-react-java-columbus-global-hyderabad-8-to-13-years-180526009415</v>
+      </c>
+      <c r="H243" t="str">
+        <v/>
+      </c>
+      <c r="I243" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244">
+        <v>243</v>
+      </c>
+      <c r="B244" t="str">
+        <v>18/5/2026, 2:39:59 pm</v>
+      </c>
+      <c r="C244" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D244" t="str">
+        <v>Walk in For Software developer (Java) &amp; Java-Technical Lead</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Al Ansari Financial Services</v>
+      </c>
+      <c r="F244" t="str">
+        <v>Hyderabad(Madhapur)</v>
+      </c>
+      <c r="G244" t="str">
+        <v>https://www.naukri.com/job-listings-walk-in-for-software-developer-java-java-technical-lead-al-ansari-financial-services-hyderabad-5-to-10-years-150526009059</v>
+      </c>
+      <c r="H244" t="str">
+        <v/>
+      </c>
+      <c r="I244" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245">
+        <v>244</v>
+      </c>
+      <c r="B245" t="str">
+        <v>18/5/2026, 2:40:07 pm</v>
+      </c>
+      <c r="C245" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D245" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Info Services</v>
+      </c>
+      <c r="F245" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G245" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-info-services-hyderabad-8-to-10-years-140526927391</v>
+      </c>
+      <c r="H245" t="str">
+        <v/>
+      </c>
+      <c r="I245" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246">
+        <v>245</v>
+      </c>
+      <c r="B246" t="str">
+        <v>18/5/2026, 2:40:45 pm</v>
+      </c>
+      <c r="C246" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D246" t="str">
+        <v>Java Full Stack Developer or Java Developer</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Qentelli</v>
+      </c>
+      <c r="F246" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G246" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-or-java-developer-qentelli-hyderabad-5-to-8-years-180526007819</v>
+      </c>
+      <c r="H246" t="str">
+        <v/>
+      </c>
+      <c r="I246" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="str">
+        <v>18/5/2026, 2:41:12 pm</v>
+      </c>
+      <c r="C247" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Java Full Stack Developer Hyderabad</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F247" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G247" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-hyderabad-infosys-hyderabad-5-to-9-years-180526002258</v>
+      </c>
+      <c r="H247" t="str">
+        <v/>
+      </c>
+      <c r="I247" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="str">
+        <v>18/5/2026, 2:41:20 pm</v>
+      </c>
+      <c r="C248" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D248" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F248" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G248" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-infosys-hyderabad-5-to-10-years-050526029661</v>
+      </c>
+      <c r="H248" t="str">
+        <v/>
+      </c>
+      <c r="I248" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="str">
+        <v>18/5/2026, 2:41:28 pm</v>
+      </c>
+      <c r="C249" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D249" t="str">
+        <v>SAP Full Stack Developer (AI Developer)</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F249" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G249" t="str">
+        <v>https://www.naukri.com/job-listings-sap-full-stack-developer-ai-developer-it-scient-hyderabad-chennai-bengaluru-10-to-14-years-180526001225</v>
+      </c>
+      <c r="H249" t="str">
+        <v/>
+      </c>
+      <c r="I249" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="str">
+        <v>18/5/2026, 2:41:37 pm</v>
+      </c>
+      <c r="C250" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D250" t="str">
+        <v>Walk-in || Solution Architect</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Ahinjay Enterprises</v>
+      </c>
+      <c r="F250" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G250" t="str">
+        <v>https://www.naukri.com/job-listings-solution-architect-ahinjay-enterprises-hyderabad-5-to-8-years-180526001217</v>
+      </c>
+      <c r="H250" t="str">
+        <v/>
+      </c>
+      <c r="I250" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="str">
+        <v>18/5/2026, 2:41:45 pm</v>
+      </c>
+      <c r="C251" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D251" t="str">
+        <v>Java Full Stack Developer | 10Yrs+ Exp | FullTime | Hyderabad</v>
+      </c>
+      <c r="E251" t="str">
+        <v>Tecnics Integration Technologies</v>
+      </c>
+      <c r="F251" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G251" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-10yrs-exp-fulltime-hyderabad-tecnics-integration-technologies-hyderabad-10-to-20-years-140526018693</v>
+      </c>
+      <c r="H251" t="str">
+        <v/>
+      </c>
+      <c r="I251" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="str">
+        <v>18/5/2026, 2:41:52 pm</v>
+      </c>
+      <c r="C252" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D252" t="str">
+        <v>Senior Java Full Stack Developer with Angular</v>
+      </c>
+      <c r="E252" t="str">
+        <v>Cognizant</v>
+      </c>
+      <c r="F252" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G252" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-with-angular-cognizant-hyderabad-8-to-13-years-140526017780</v>
+      </c>
+      <c r="H252" t="str">
+        <v/>
+      </c>
+      <c r="I252" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253">
+        <v>252</v>
+      </c>
+      <c r="B253" t="str">
+        <v>18/5/2026, 2:42:00 pm</v>
+      </c>
+      <c r="C253" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D253" t="str">
+        <v>.NET Full Stack Developer</v>
+      </c>
+      <c r="E253" t="str">
+        <v>S&amp;P Global Market Intelligence</v>
+      </c>
+      <c r="F253" t="str">
+        <v>Hyderabad, Ahmedabad</v>
+      </c>
+      <c r="G253" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-s-p-capital-iq-india-pvt-ltd-hyderabad-ahmedabad-5-to-8-years-130526941821</v>
+      </c>
+      <c r="H253" t="str">
+        <v/>
+      </c>
+      <c r="I253" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I226"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I253"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add job cleanup script to remove stale entries and rebuild Excel
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I85"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2791,16 +2791,103 @@
         <v>Naukri quick-apply (auto)</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="str">
+        <v>19/5/2026, 6:05:20 pm</v>
+      </c>
+      <c r="C83" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Full Stack Developer - Nodejs ReactJS AngularJS</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Cerebra</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G83" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-nodejs-reactjs-angularjs-cerebra-hyderabad-chennai-bengaluru-4-to-8-years-170426010247</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="str">
+        <v>19/5/2026, 6:06:17 pm</v>
+      </c>
+      <c r="C84" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Software Engineer 2 .Net Developer</v>
+      </c>
+      <c r="E84" t="str">
+        <v>E-Ring</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Hyderabad(Madhapur)</v>
+      </c>
+      <c r="G84" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-2-net-developer-e-ring-hyderabad-3-to-6-years-180526024209</v>
+      </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+      <c r="I84" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="str">
+        <v>19/5/2026, 6:09:04 pm</v>
+      </c>
+      <c r="C85" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Azure dot net full stack developer</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G85" t="str">
+        <v>https://www.naukri.com/job-listings-azure-dot-net-full-stack-developer-tata-consultancy-services-hyderabad-pune-bengaluru-4-to-9-years-190526010797</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I85"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I375"/>
+  <dimension ref="A1:I388"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -13688,9 +13775,386 @@
         <v>External — apply manually</v>
       </c>
     </row>
+    <row r="376">
+      <c r="A376">
+        <v>375</v>
+      </c>
+      <c r="B376" t="str">
+        <v>19/5/2026, 6:03:13 pm</v>
+      </c>
+      <c r="C376" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D376" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E376" t="str">
+        <v>Ahsan Solutions</v>
+      </c>
+      <c r="F376" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G376" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-ahsan-solutions-hyderabad-2-to-3-years-130526500581</v>
+      </c>
+      <c r="H376" t="str">
+        <v>https://ahsansolutions.com/careers</v>
+      </c>
+      <c r="I376" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377">
+        <v>376</v>
+      </c>
+      <c r="B377" t="str">
+        <v>19/5/2026, 6:04:13 pm</v>
+      </c>
+      <c r="C377" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D377" t="str">
+        <v>Full Stack Developer - MEAN Stack</v>
+      </c>
+      <c r="E377" t="str">
+        <v>Smartify Software Solutions</v>
+      </c>
+      <c r="F377" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G377" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-mean-stack-smartify-software-solutions-llp-hyderabad-2-to-4-years-180526506889</v>
+      </c>
+      <c r="H377" t="str">
+        <v>https://smartifysol.com/jobs/full-stack-developer-mean-stack-job/</v>
+      </c>
+      <c r="I377" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378">
+        <v>377</v>
+      </c>
+      <c r="B378" t="str">
+        <v>19/5/2026, 6:04:34 pm</v>
+      </c>
+      <c r="C378" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D378" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E378" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F378" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G378" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-190526921402</v>
+      </c>
+      <c r="H378" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500971-S2014336_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I378" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379">
+        <v>378</v>
+      </c>
+      <c r="B379" t="str">
+        <v>19/5/2026, 6:04:38 pm</v>
+      </c>
+      <c r="C379" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E379" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F379" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G379" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-180526920532</v>
+      </c>
+      <c r="H379" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5307647-S1937329_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I379" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380">
+        <v>379</v>
+      </c>
+      <c r="B380" t="str">
+        <v>19/5/2026, 6:04:53 pm</v>
+      </c>
+      <c r="C380" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D380" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E380" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F380" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G380" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-190526922483</v>
+      </c>
+      <c r="H380" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500995-S2014322_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I380" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381">
+        <v>380</v>
+      </c>
+      <c r="B381" t="str">
+        <v>19/5/2026, 6:04:59 pm</v>
+      </c>
+      <c r="C381" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E381" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F381" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G381" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-180526921255</v>
+      </c>
+      <c r="H381" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-4913986-S1933573_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I381" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382">
+        <v>381</v>
+      </c>
+      <c r="B382" t="str">
+        <v>19/5/2026, 6:05:06 pm</v>
+      </c>
+      <c r="C382" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="E382" t="str">
+        <v>Alter Domus</v>
+      </c>
+      <c r="F382" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G382" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-alter-domus-hyderabad-2-to-5-years-180526506453</v>
+      </c>
+      <c r="H382" t="str">
+        <v>https://careers.alterdomus.com/en/job/hyderabad/software-engineer/38735/38486868032</v>
+      </c>
+      <c r="I382" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383">
+        <v>382</v>
+      </c>
+      <c r="B383" t="str">
+        <v>19/5/2026, 6:05:10 pm</v>
+      </c>
+      <c r="C383" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E383" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F383" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G383" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-180526920820</v>
+      </c>
+      <c r="H383" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobsearch</v>
+      </c>
+      <c r="I383" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384">
+        <v>383</v>
+      </c>
+      <c r="B384" t="str">
+        <v>19/5/2026, 6:05:25 pm</v>
+      </c>
+      <c r="C384" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Software Engineer - Java Full Stack Developer</v>
+      </c>
+      <c r="E384" t="str">
+        <v>Dtcc</v>
+      </c>
+      <c r="F384" t="str">
+        <v>Hyderabad, Chennai</v>
+      </c>
+      <c r="G384" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-java-full-stack-developer-dtcc-hyderabad-chennai-3-to-5-years-180526918084</v>
+      </c>
+      <c r="H384" t="str">
+        <v>https://ebxr.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/213583/</v>
+      </c>
+      <c r="I384" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385">
+        <v>384</v>
+      </c>
+      <c r="B385" t="str">
+        <v>19/5/2026, 6:05:31 pm</v>
+      </c>
+      <c r="C385" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D385" t="str">
+        <v>Dot Net Full Stack Developer</v>
+      </c>
+      <c r="E385" t="str">
+        <v>LPL Financial</v>
+      </c>
+      <c r="F385" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G385" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-lpl-financial-hyderabad-3-to-8-years-190526501144</v>
+      </c>
+      <c r="H385" t="str">
+        <v>https://lplfinancial.wd1.myworkdayjobs.com/en-US/India_Ext/job/Hyderabad/XMLNAME-Net-Full-Stack-Developer_R-048972</v>
+      </c>
+      <c r="I385" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386">
+        <v>385</v>
+      </c>
+      <c r="B386" t="str">
+        <v>19/5/2026, 6:08:14 pm</v>
+      </c>
+      <c r="C386" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D386" t="str">
+        <v>Senior .Net Full Stack Developer</v>
+      </c>
+      <c r="E386" t="str">
+        <v>LPL Financial</v>
+      </c>
+      <c r="F386" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G386" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-lpl-financial-hyderabad-6-to-11-years-190526500583</v>
+      </c>
+      <c r="H386" t="str">
+        <v>https://lplfinancial.wd1.myworkdayjobs.com/en-US/India_Ext/job/Hyderabad/Senior-Net-Full-Stack-Developer_R-048971</v>
+      </c>
+      <c r="I386" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387">
+        <v>386</v>
+      </c>
+      <c r="B387" t="str">
+        <v>19/5/2026, 6:08:19 pm</v>
+      </c>
+      <c r="C387" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Senior .Net Full Stack Developer Senior</v>
+      </c>
+      <c r="E387" t="str">
+        <v>LPL Financial</v>
+      </c>
+      <c r="F387" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G387" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-senior-lpl-financial-hyderabad-6-to-11-years-190526500582</v>
+      </c>
+      <c r="H387" t="str">
+        <v>https://lplfinancial.wd1.myworkdayjobs.com/en-US/India_Ext/job/Hyderabad/Senior-Net-Full-Stack-DeveloperSenior_R-050123</v>
+      </c>
+      <c r="I387" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388">
+        <v>387</v>
+      </c>
+      <c r="B388" t="str">
+        <v>19/5/2026, 6:09:09 pm</v>
+      </c>
+      <c r="C388" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Senior Full Stack Developer (Angular / React &amp; Java)</v>
+      </c>
+      <c r="E388" t="str">
+        <v>Columbus Global</v>
+      </c>
+      <c r="F388" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G388" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-angular-react-java-columbus-global-services-india-pvt-ltd-hyderabad-5-to-10-years-180526504104</v>
+      </c>
+      <c r="H388" t="str">
+        <v>https://careers-india.columbusglobal.com/jobs/7739227-senior-full-stack-developer-angular-react-java</v>
+      </c>
+      <c r="I388" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I375"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I388"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -13748,7 +14212,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I253"/>
+  <dimension ref="A1:I275"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -21098,9 +21562,647 @@
         <v>unknown_state</v>
       </c>
     </row>
+    <row r="254">
+      <c r="A254">
+        <v>253</v>
+      </c>
+      <c r="B254" t="str">
+        <v>19/5/2026, 6:03:41 pm</v>
+      </c>
+      <c r="C254" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D254" t="str">
+        <v>Angular/PHP Full Stack Developer</v>
+      </c>
+      <c r="E254" t="str">
+        <v>Sune Solutions</v>
+      </c>
+      <c r="F254" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G254" t="str">
+        <v>https://www.naukri.com/job-listings-angular-php-full-stack-developer-sune-solutions-hyderabad-2-to-5-years-180526011392</v>
+      </c>
+      <c r="H254" t="str">
+        <v/>
+      </c>
+      <c r="I254" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255">
+        <v>254</v>
+      </c>
+      <c r="B255" t="str">
+        <v>19/5/2026, 6:04:08 pm</v>
+      </c>
+      <c r="C255" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D255" t="str">
+        <v>Senior Associate-.NET Full Stack Developer</v>
+      </c>
+      <c r="E255" t="str">
+        <v>Genpact</v>
+      </c>
+      <c r="F255" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G255" t="str">
+        <v>https://www.naukri.com/job-listings-senior-associate-net-full-stack-developer-genpact-hyderabad-1-to-3-years-190526018151</v>
+      </c>
+      <c r="H255" t="str">
+        <v/>
+      </c>
+      <c r="I255" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256">
+        <v>255</v>
+      </c>
+      <c r="B256" t="str">
+        <v>19/5/2026, 6:04:21 pm</v>
+      </c>
+      <c r="C256" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D256" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E256" t="str">
+        <v>Service Industry</v>
+      </c>
+      <c r="F256" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G256" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-anlage-infotech-hyderabad-pune-bengaluru-2-to-7-years-180526029445</v>
+      </c>
+      <c r="H256" t="str">
+        <v/>
+      </c>
+      <c r="I256" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257">
+        <v>256</v>
+      </c>
+      <c r="B257" t="str">
+        <v>19/5/2026, 6:04:29 pm</v>
+      </c>
+      <c r="C257" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D257" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E257" t="str">
+        <v>client of Anlage</v>
+      </c>
+      <c r="F257" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G257" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-anlage-infotech-hyderabad-chennai-bengaluru-2-to-5-years-180526024360</v>
+      </c>
+      <c r="H257" t="str">
+        <v/>
+      </c>
+      <c r="I257" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258">
+        <v>257</v>
+      </c>
+      <c r="B258" t="str">
+        <v>19/5/2026, 6:04:46 pm</v>
+      </c>
+      <c r="C258" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D258" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="E258" t="str">
+        <v>GE VERNOVA</v>
+      </c>
+      <c r="F258" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G258" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-ge-renewable-energy-technologies-private-limited-hyderabad-2-to-5-years-190526925986</v>
+      </c>
+      <c r="H258" t="str">
+        <v/>
+      </c>
+      <c r="I258" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259">
+        <v>258</v>
+      </c>
+      <c r="B259" t="str">
+        <v>19/5/2026, 6:05:40 pm</v>
+      </c>
+      <c r="C259" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D259" t="str">
+        <v>Full Stack .Net Developer</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Ray Business Technologies</v>
+      </c>
+      <c r="F259" t="str">
+        <v>Hyderabad(Madhapur), Indore</v>
+      </c>
+      <c r="G259" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-net-developer-ray-business-technologies-indore-hyderabad-6-to-10-years-110526034545</v>
+      </c>
+      <c r="H259" t="str">
+        <v/>
+      </c>
+      <c r="I259" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260">
+        <v>259</v>
+      </c>
+      <c r="B260" t="str">
+        <v>19/5/2026, 6:06:07 pm</v>
+      </c>
+      <c r="C260" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D260" t="str">
+        <v>Java Full Stack Developer (React JS +Node jS)</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F260" t="str">
+        <v>Hyderabad, Mumbai (All Areas), Kolkata</v>
+      </c>
+      <c r="G260" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-react-js-node-js-tata-consultancy-services-kolkata-hyderabad-mumbai-all-areas-5-to-10-years-150526030700</v>
+      </c>
+      <c r="H260" t="str">
+        <v/>
+      </c>
+      <c r="I260" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261">
+        <v>260</v>
+      </c>
+      <c r="B261" t="str">
+        <v>19/5/2026, 6:06:25 pm</v>
+      </c>
+      <c r="C261" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D261" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E261" t="str">
+        <v>Giant MNC</v>
+      </c>
+      <c r="F261" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G261" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-anlage-infotech-hyderabad-pune-bengaluru-3-to-7-years-180526028678</v>
+      </c>
+      <c r="H261" t="str">
+        <v/>
+      </c>
+      <c r="I261" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262">
+        <v>261</v>
+      </c>
+      <c r="B262" t="str">
+        <v>19/5/2026, 6:06:52 pm</v>
+      </c>
+      <c r="C262" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D262" t="str">
+        <v>Senior Java Full Stack Developer (Java, React, Azure)</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Conduent</v>
+      </c>
+      <c r="F262" t="str">
+        <v>Hybrid - Hyderabad, Noida, Bengaluru</v>
+      </c>
+      <c r="G262" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-java-react-azure-conduent-noida-hyderabad-bengaluru-7-to-10-years-190526017756</v>
+      </c>
+      <c r="H262" t="str">
+        <v/>
+      </c>
+      <c r="I262" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263">
+        <v>262</v>
+      </c>
+      <c r="B263" t="str">
+        <v>19/5/2026, 6:07:19 pm</v>
+      </c>
+      <c r="C263" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D263" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E263" t="str">
+        <v>MNC Group</v>
+      </c>
+      <c r="F263" t="str">
+        <v>Hybrid - Hyderabad, Mumbai (All Areas), Bengaluru</v>
+      </c>
+      <c r="G263" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-professional-connect-hyderabad-bengaluru-mumbai-all-areas-6-to-11-years-190526013340</v>
+      </c>
+      <c r="H263" t="str">
+        <v/>
+      </c>
+      <c r="I263" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264">
+        <v>263</v>
+      </c>
+      <c r="B264" t="str">
+        <v>19/5/2026, 6:07:46 pm</v>
+      </c>
+      <c r="C264" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D264" t="str">
+        <v>Python Full stack Developer - Remote Opportunity</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Siro Clinpharm</v>
+      </c>
+      <c r="F264" t="str">
+        <v>Hyderabad, Noida, Bengaluru</v>
+      </c>
+      <c r="G264" t="str">
+        <v>https://www.naukri.com/job-listings-python-full-stack-developer-remote-opportunity-siro-clinpharm-noida-hyderabad-bengaluru-7-to-12-years-180526013108</v>
+      </c>
+      <c r="H264" t="str">
+        <v/>
+      </c>
+      <c r="I264" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265">
+        <v>264</v>
+      </c>
+      <c r="B265" t="str">
+        <v>19/5/2026, 6:07:54 pm</v>
+      </c>
+      <c r="C265" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D265" t="str">
+        <v>Java Full Stack Developer (React.js is must)</v>
+      </c>
+      <c r="E265" t="str">
+        <v>Reveille Technologies</v>
+      </c>
+      <c r="F265" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G265" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-react-js-is-must-reveille-technologies-hyderabad-chennai-bengaluru-7-to-11-years-190526023099</v>
+      </c>
+      <c r="H265" t="str">
+        <v/>
+      </c>
+      <c r="I265" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266">
+        <v>265</v>
+      </c>
+      <c r="B266" t="str">
+        <v>19/5/2026, 6:08:02 pm</v>
+      </c>
+      <c r="C266" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D266" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E266" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F266" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G266" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-11-years-180526023600</v>
+      </c>
+      <c r="H266" t="str">
+        <v/>
+      </c>
+      <c r="I266" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267">
+        <v>266</v>
+      </c>
+      <c r="B267" t="str">
+        <v>19/5/2026, 6:08:10 pm</v>
+      </c>
+      <c r="C267" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D267" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E267" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F267" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G267" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-infosys-hyderabad-chennai-bengaluru-5-to-10-years-200326026193</v>
+      </c>
+      <c r="H267" t="str">
+        <v/>
+      </c>
+      <c r="I267" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268">
+        <v>267</v>
+      </c>
+      <c r="B268" t="str">
+        <v>19/5/2026, 6:08:46 pm</v>
+      </c>
+      <c r="C268" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D268" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E268" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F268" t="str">
+        <v>Hyderabad, Kochi, Chennai</v>
+      </c>
+      <c r="G268" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-wipro-kochi-hyderabad-chennai-5-to-8-years-190526030182</v>
+      </c>
+      <c r="H268" t="str">
+        <v/>
+      </c>
+      <c r="I268" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269">
+        <v>268</v>
+      </c>
+      <c r="B269" t="str">
+        <v>19/5/2026, 6:08:54 pm</v>
+      </c>
+      <c r="C269" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D269" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E269" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F269" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G269" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-5-to-10-years-190526025840</v>
+      </c>
+      <c r="H269" t="str">
+        <v/>
+      </c>
+      <c r="I269" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270">
+        <v>269</v>
+      </c>
+      <c r="B270" t="str">
+        <v>19/5/2026, 6:09:39 pm</v>
+      </c>
+      <c r="C270" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D270" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E270" t="str">
+        <v>Hexaware Technologies</v>
+      </c>
+      <c r="F270" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G270" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-hexaware-technologies-hyderabad-chennai-bengaluru-6-to-10-years-180526027670</v>
+      </c>
+      <c r="H270" t="str">
+        <v/>
+      </c>
+      <c r="I270" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271">
+        <v>270</v>
+      </c>
+      <c r="B271" t="str">
+        <v>19/5/2026, 6:09:46 pm</v>
+      </c>
+      <c r="C271" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D271" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E271" t="str">
+        <v>CGI</v>
+      </c>
+      <c r="F271" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G271" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-cgi-hyderabad-chennai-bengaluru-5-to-9-years-180526012613</v>
+      </c>
+      <c r="H271" t="str">
+        <v/>
+      </c>
+      <c r="I271" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272">
+        <v>271</v>
+      </c>
+      <c r="B272" t="str">
+        <v>19/5/2026, 6:09:50 pm</v>
+      </c>
+      <c r="C272" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D272" t="str">
+        <v>Walk-in || Solution Architect</v>
+      </c>
+      <c r="E272" t="str">
+        <v>Ahinjay Enterprises</v>
+      </c>
+      <c r="F272" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G272" t="str">
+        <v>https://www.naukri.com/job-listings-solution-architect-ahinjay-enterprises-hyderabad-10-to-15-years-180526001217</v>
+      </c>
+      <c r="H272" t="str">
+        <v/>
+      </c>
+      <c r="I272" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273">
+        <v>272</v>
+      </c>
+      <c r="B273" t="str">
+        <v>19/5/2026, 6:09:54 pm</v>
+      </c>
+      <c r="C273" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D273" t="str">
+        <v>Walk-in || UX and UI Designer</v>
+      </c>
+      <c r="E273" t="str">
+        <v>Tekreant</v>
+      </c>
+      <c r="F273" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G273" t="str">
+        <v>https://www.naukri.com/job-listings-ux-and-ui-designer-tekreant-hyderabad-3-to-6-years-190526020618</v>
+      </c>
+      <c r="H273" t="str">
+        <v/>
+      </c>
+      <c r="I273" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274">
+        <v>273</v>
+      </c>
+      <c r="B274" t="str">
+        <v>19/5/2026, 6:10:21 pm</v>
+      </c>
+      <c r="C274" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D274" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E274" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F274" t="str">
+        <v>Hyderabad, Mumbai (All Areas), Bengaluru</v>
+      </c>
+      <c r="G274" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-bengaluru-mumbai-all-areas-5-to-10-years-180526025203</v>
+      </c>
+      <c r="H274" t="str">
+        <v/>
+      </c>
+      <c r="I274" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275">
+        <v>274</v>
+      </c>
+      <c r="B275" t="str">
+        <v>19/5/2026, 6:10:48 pm</v>
+      </c>
+      <c r="C275" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D275" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E275" t="str">
+        <v>Saransh Software Solutions</v>
+      </c>
+      <c r="F275" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G275" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-saransh-software-solutions-hyderabad-6-to-11-years-300326014395</v>
+      </c>
+      <c r="H275" t="str">
+        <v/>
+      </c>
+      <c r="I275" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I253"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I275"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job applications spreadsheet with latest data
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I92"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -2878,16 +2878,219 @@
         <v>Naukri quick-apply (auto)</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="str">
+        <v>27/5/2026, 11:33:47 am</v>
+      </c>
+      <c r="C86" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Talent Acquisition Specialist - Product Hiring</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Techolution</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Hybrid - Hyderabad(Nanakramguda)</v>
+      </c>
+      <c r="G86" t="str">
+        <v>https://www.naukri.com/job-listings-talent-acquisition-specialist-product-hiring-techolution-hyderabad-2-to-7-years-250526036447</v>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="str">
+        <v>27/5/2026, 11:33:57 am</v>
+      </c>
+      <c r="C87" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Talent Acquisition Specialist / IT Recruiter - Product Hiring</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Techolution</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Hybrid - Hyderabad(Nanakramguda)</v>
+      </c>
+      <c r="G87" t="str">
+        <v>https://www.naukri.com/job-listings-talent-acquisition-specialist-it-recruiter-product-hiring-techolution-hyderabad-2-to-7-years-240326016513</v>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="str">
+        <v>27/5/2026, 11:35:31 am</v>
+      </c>
+      <c r="C88" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D88" t="str">
+        <v>.Net Fullstack developer(AI)</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Top MNC Company</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Hyderabad, Kolkata, Chennai</v>
+      </c>
+      <c r="G88" t="str">
+        <v>https://www.naukri.com/job-listings-net-fullstack-developer-ai-sigma-allied-services-kolkata-hyderabad-chennai-2-to-5-years-050526039171</v>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+      <c r="I88" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="str">
+        <v>27/5/2026, 11:36:59 am</v>
+      </c>
+      <c r="C89" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Full Stack with AI Developer Opening with CAPCO</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Capco</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Hybrid - Hyderabad, Gurugram, Bengaluru</v>
+      </c>
+      <c r="G89" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-with-ai-developer-opening-with-capco-capco-hyderabad-gurugram-bengaluru-7-to-12-years-250326020186</v>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="str">
+        <v>27/5/2026, 11:41:37 am</v>
+      </c>
+      <c r="C90" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D90" t="str">
+        <v>AI Full Stack Developer</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Tata Consultancy Services(TCS)</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G90" t="str">
+        <v>https://www.naukri.com/job-listings-ai-full-stack-developer-it-scient-hyderabad-chennai-bengaluru-11-to-21-years-220526012278</v>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="str">
+        <v>27/5/2026, 11:41:48 am</v>
+      </c>
+      <c r="C91" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D91" t="str">
+        <v>AI Full Stack Developer</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Tata Consultancy Services(TCS)</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G91" t="str">
+        <v>https://www.naukri.com/job-listings-ai-full-stack-developer-it-scient-hyderabad-chennai-bengaluru-12-to-21-years-220526012266</v>
+      </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="str">
+        <v>27/5/2026, 11:42:45 am</v>
+      </c>
+      <c r="C92" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Sr. Full Stack Developer (Python) &amp; Generative AI</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Programmers io</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="G92" t="str">
+        <v>https://www.naukri.com/job-listings-sr-full-stack-developer-python-generative-ai-programmers-io-hyderabad-6-to-10-years-250526007226</v>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v>Naukri quick-apply (auto)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I92"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I388"/>
+  <dimension ref="A1:I423"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -14152,9 +14355,1024 @@
         <v>External — apply manually</v>
       </c>
     </row>
+    <row r="389">
+      <c r="A389">
+        <v>388</v>
+      </c>
+      <c r="B389" t="str">
+        <v>27/5/2026, 11:33:20 am</v>
+      </c>
+      <c r="C389" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E389" t="str">
+        <v>Qapitol Qa</v>
+      </c>
+      <c r="F389" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G389" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-qapitol-qa-services-private-limited-hyderabad-2-to-6-years-070526500598</v>
+      </c>
+      <c r="H389" t="str">
+        <v>https://www.qapitol.com/career-openings?job_id=z5G7h3l6a1kMvyS65NP3c97Qcs1ODABQxRTTkNdeyNY=</v>
+      </c>
+      <c r="I389" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390">
+        <v>389</v>
+      </c>
+      <c r="B390" t="str">
+        <v>27/5/2026, 11:33:24 am</v>
+      </c>
+      <c r="C390" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D390" t="str">
+        <v>Dot Net full stack Developer</v>
+      </c>
+      <c r="E390" t="str">
+        <v>Stack Digital</v>
+      </c>
+      <c r="F390" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G390" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-stack-digital-warangal-hyderabad-nizamabad-2-to-7-years-260526506335</v>
+      </c>
+      <c r="H390" t="str">
+        <v>https://www.gostack.co.in/careers?job_id=z5G7h3l6a1kMvyS65NP3cyd6dREvRylrPiaSO4ktG8k=</v>
+      </c>
+      <c r="I390" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391">
+        <v>390</v>
+      </c>
+      <c r="B391" t="str">
+        <v>27/5/2026, 11:33:28 am</v>
+      </c>
+      <c r="C391" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Net Full stack Developer - MDM custom application development</v>
+      </c>
+      <c r="E391" t="str">
+        <v>Stack Digital</v>
+      </c>
+      <c r="F391" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G391" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-mdm-custom-application-development-stack-digital-warangal-hyderabad-nizamabad-2-to-7-years-260526506334</v>
+      </c>
+      <c r="H391" t="str">
+        <v>https://www.gostack.co.in/careers?job_id=z5G7h3l6a1kMvyS65NP3c7IG9S22Erg8y1F-OB8k3YE=</v>
+      </c>
+      <c r="I391" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392">
+        <v>391</v>
+      </c>
+      <c r="B392" t="str">
+        <v>27/5/2026, 11:34:02 am</v>
+      </c>
+      <c r="C392" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E392" t="str">
+        <v>Multicloud4u Technologies</v>
+      </c>
+      <c r="F392" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G392" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-multicloud4u-technologies-warangal-hyderabad-nizamabad-2-to-7-years-260526502579</v>
+      </c>
+      <c r="H392" t="str">
+        <v>https://www.5thir.com/jobs/job_detail_page.aspx?jobid=JOB_3B8VZC8VVUXVOFWUWM27B9QSZ&amp;refcode=966856&amp;referrar=</v>
+      </c>
+      <c r="I392" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393">
+        <v>392</v>
+      </c>
+      <c r="B393" t="str">
+        <v>27/5/2026, 11:34:34 am</v>
+      </c>
+      <c r="C393" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D393" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E393" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F393" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G393" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-250526922257</v>
+      </c>
+      <c r="H393" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5264904-S1928195_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I393" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394">
+        <v>393</v>
+      </c>
+      <c r="B394" t="str">
+        <v>27/5/2026, 11:35:07 am</v>
+      </c>
+      <c r="C394" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Full Stack Software Engineer</v>
+      </c>
+      <c r="E394" t="str">
+        <v>Amgen Inc</v>
+      </c>
+      <c r="F394" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G394" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-software-engineer-amgen-inc-hyderabad-2-to-6-years-250526934992</v>
+      </c>
+      <c r="H394" t="str">
+        <v>https://careers.amgen.com/en/job/-/-/87/84320467600?source=rd_naukri&amp;utm_source=naukri.com&amp;utm_medium=job_posting&amp;utm_campaign=Healthcare_General&amp;utm_content=job_board&amp;utm_term=402434614&amp;ss=paid</v>
+      </c>
+      <c r="I394" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395">
+        <v>394</v>
+      </c>
+      <c r="B395" t="str">
+        <v>27/5/2026, 11:35:11 am</v>
+      </c>
+      <c r="C395" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E395" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F395" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G395" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-200526940494</v>
+      </c>
+      <c r="H395" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5263241-S1945727_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I395" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396">
+        <v>395</v>
+      </c>
+      <c r="B396" t="str">
+        <v>27/5/2026, 11:35:15 am</v>
+      </c>
+      <c r="C396" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D396" t="str">
+        <v>Software Development Engineer</v>
+      </c>
+      <c r="E396" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F396" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G396" t="str">
+        <v>https://www.naukri.com/job-listings-software-development-engineer-accenture-solutions-pvt-ltd-hyderabad-1-to-4-years-250526925858</v>
+      </c>
+      <c r="H396" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5054455-S1900617_en&amp;title=Software+Development+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I396" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397">
+        <v>396</v>
+      </c>
+      <c r="B397" t="str">
+        <v>27/5/2026, 11:35:35 am</v>
+      </c>
+      <c r="C397" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D397" t="str">
+        <v>Custom Software Engineer</v>
+      </c>
+      <c r="E397" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F397" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G397" t="str">
+        <v>https://www.naukri.com/job-listings-custom-software-engineer-accenture-solutions-pvt-ltd-hyderabad-2-to-5-years-190526921227</v>
+      </c>
+      <c r="H397" t="str">
+        <v>https://www.accenture.com/in-en/careers/jobdetails?id=ATCI-5500972-S2014297_en&amp;title=Custom+Software+Engineer&amp;SRC=RECNau</v>
+      </c>
+      <c r="I397" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398">
+        <v>397</v>
+      </c>
+      <c r="B398" t="str">
+        <v>27/5/2026, 11:35:49 am</v>
+      </c>
+      <c r="C398" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D398" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E398" t="str">
+        <v>Hitachi Digital Services</v>
+      </c>
+      <c r="F398" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G398" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-hitachi-digital-services-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-3-to-6-years-290425503662</v>
+      </c>
+      <c r="H398" t="str">
+        <v>https://hitachidigital.com/careers/job-details/?jid=7922582002&amp;gh_jid=7922582002&amp;gh_src=e88a2f692us</v>
+      </c>
+      <c r="I398" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399">
+        <v>398</v>
+      </c>
+      <c r="B399" t="str">
+        <v>27/5/2026, 11:35:54 am</v>
+      </c>
+      <c r="C399" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D399" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E399" t="str">
+        <v>Tech Stalwart Solution</v>
+      </c>
+      <c r="F399" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G399" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-tech-stalwart-solution-private-limited-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-3-to-8-years-020525500736</v>
+      </c>
+      <c r="H399" t="str">
+        <v>https://techstalwartsolution.com/career.html?job_id=z5G7h3l6a1kMvyS65NP3c7EFj2l9OPAymHLKDgbgaKI=</v>
+      </c>
+      <c r="I399" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400">
+        <v>399</v>
+      </c>
+      <c r="B400" t="str">
+        <v>27/5/2026, 11:36:01 am</v>
+      </c>
+      <c r="C400" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E400" t="str">
+        <v>IDESLABS</v>
+      </c>
+      <c r="F400" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G400" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-ideslabs-private-limited-hyderabad-3-to-10-years-061223502249</v>
+      </c>
+      <c r="H400" t="str">
+        <v>https://ideslabs.com/current-openings.php?job_id=z5G7h3l6a1kMvyS65NP3c63JgKChSqNBLGwiFnNQpY8=</v>
+      </c>
+      <c r="I400" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401">
+        <v>400</v>
+      </c>
+      <c r="B401" t="str">
+        <v>27/5/2026, 11:36:19 am</v>
+      </c>
+      <c r="C401" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E401" t="str">
+        <v>Acme Services</v>
+      </c>
+      <c r="F401" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G401" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-acme-services-hyderabad-2-to-7-years-210223501221</v>
+      </c>
+      <c r="H401" t="str">
+        <v>https://www.acme-services.in/current-openings/?job_id=z5G7h3l6a1kMvyS65NP3c0s3vqfcSZnVm4gAy8_Pyck=</v>
+      </c>
+      <c r="I401" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402">
+        <v>401</v>
+      </c>
+      <c r="B402" t="str">
+        <v>27/5/2026, 11:36:42 am</v>
+      </c>
+      <c r="C402" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D402" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E402" t="str">
+        <v>Triad Square Infosec</v>
+      </c>
+      <c r="F402" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G402" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-triad-square-infotec-pvt-ltd-hyderabad-5-to-10-years-270625500180</v>
+      </c>
+      <c r="H402" t="str">
+        <v>https://triadsquare.com/career/</v>
+      </c>
+      <c r="I402" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403">
+        <v>402</v>
+      </c>
+      <c r="B403" t="str">
+        <v>27/5/2026, 11:37:05 am</v>
+      </c>
+      <c r="C403" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E403" t="str">
+        <v>Tech Stalwart Solution</v>
+      </c>
+      <c r="F403" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G403" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-tech-stalwart-solution-private-limited-hyderabad-5-to-7-years-100325500811</v>
+      </c>
+      <c r="H403" t="str">
+        <v>https://jobsapi.ceipal.com/APISource/v4/index.html?job_id=z5G7h3l6a1kMvyS65NP3c3BNeXWSVwa3oQQovzPEcTs=</v>
+      </c>
+      <c r="I403" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404">
+        <v>403</v>
+      </c>
+      <c r="B404" t="str">
+        <v>27/5/2026, 11:37:11 am</v>
+      </c>
+      <c r="C404" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E404" t="str">
+        <v>LLP S3bglobal Technologies</v>
+      </c>
+      <c r="F404" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G404" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-s3b-global-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-5-to-9-years-300724502066</v>
+      </c>
+      <c r="H404" t="str">
+        <v>https://s3bglobal.com/careers_v1/?job_id=z5G7h3l6a1kMvyS65NP3cx0RYVs4AK9V8r2dHw9tToM=</v>
+      </c>
+      <c r="I404" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405">
+        <v>404</v>
+      </c>
+      <c r="B405" t="str">
+        <v>27/5/2026, 11:38:26 am</v>
+      </c>
+      <c r="C405" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D405" t="str">
+        <v>Senior Java Full Stack Developer</v>
+      </c>
+      <c r="E405" t="str">
+        <v>Whopper Technologies</v>
+      </c>
+      <c r="F405" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G405" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-whopper-technologies-hyderabad-5-to-9-years-270325501262</v>
+      </c>
+      <c r="H405" t="str">
+        <v>chrome-error://chromewebdata/</v>
+      </c>
+      <c r="I405" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406">
+        <v>405</v>
+      </c>
+      <c r="B406" t="str">
+        <v>27/5/2026, 11:38:36 am</v>
+      </c>
+      <c r="C406" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Senior NET Full Stack Developer Digital</v>
+      </c>
+      <c r="E406" t="str">
+        <v>Feuji Inc</v>
+      </c>
+      <c r="F406" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G406" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-digital-feuji-warangal-hyderabad-nizamabad-8-to-12-years-270226503690</v>
+      </c>
+      <c r="H406" t="str">
+        <v>https://www.feuji.com/careers?job_id=z5G7h3l6a1kMvyS65NP3c1qC8I2GPSp1_MZ7Dk3Tc1E%3D</v>
+      </c>
+      <c r="I406" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407">
+        <v>406</v>
+      </c>
+      <c r="B407" t="str">
+        <v>27/5/2026, 11:38:43 am</v>
+      </c>
+      <c r="C407" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D407" t="str">
+        <v>Lead Net Full Stack Developer</v>
+      </c>
+      <c r="E407" t="str">
+        <v>Feuji Inc</v>
+      </c>
+      <c r="F407" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G407" t="str">
+        <v>https://www.naukri.com/job-listings-lead-net-full-stack-developer-feuji-warangal-hyderabad-nizamabad-3-to-12-years-270226503689</v>
+      </c>
+      <c r="H407" t="str">
+        <v>https://www.feuji.com/careers?job_id=z5G7h3l6a1kMvyS65NP3c7iNoDthQI9Xe10BnDmm37A%3D</v>
+      </c>
+      <c r="I407" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408">
+        <v>407</v>
+      </c>
+      <c r="B408" t="str">
+        <v>27/5/2026, 11:38:50 am</v>
+      </c>
+      <c r="C408" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D408" t="str">
+        <v>Net Full Stack Developer</v>
+      </c>
+      <c r="E408" t="str">
+        <v>Feuji Inc</v>
+      </c>
+      <c r="F408" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G408" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-feuji-warangal-hyderabad-nizamabad-5-to-10-years-270226503687</v>
+      </c>
+      <c r="H408" t="str">
+        <v>https://www.feuji.com/careers?job_id=z5G7h3l6a1kMvyS65NP3c_NTSS2YmZ7cxmKc52pTMGo%3D</v>
+      </c>
+      <c r="I408" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409">
+        <v>408</v>
+      </c>
+      <c r="B409" t="str">
+        <v>27/5/2026, 11:39:02 am</v>
+      </c>
+      <c r="C409" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D409" t="str">
+        <v>Full Stack Web Developer</v>
+      </c>
+      <c r="E409" t="str">
+        <v>Nfosoft Innovation</v>
+      </c>
+      <c r="F409" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G409" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-web-developer-nfosoft-innovations-pvt-ltd-hyderabad-2-to-6-years-270225501800</v>
+      </c>
+      <c r="H409" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-web-developer-nfosoft-innovations-pvt-ltd-hyderabad-2-to-6-years-270225501800</v>
+      </c>
+      <c r="I409" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410">
+        <v>409</v>
+      </c>
+      <c r="B410" t="str">
+        <v>27/5/2026, 11:39:09 am</v>
+      </c>
+      <c r="C410" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D410" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E410" t="str">
+        <v>Ice.com</v>
+      </c>
+      <c r="F410" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G410" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-ice-com-hyderabad-5-to-6-years-270126503091</v>
+      </c>
+      <c r="H410" t="str">
+        <v>https://careers.ice.com/jobs/12020?lang=en-us</v>
+      </c>
+      <c r="I410" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411">
+        <v>410</v>
+      </c>
+      <c r="B411" t="str">
+        <v>27/5/2026, 11:39:14 am</v>
+      </c>
+      <c r="C411" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D411" t="str">
+        <v>Java full stack Developer</v>
+      </c>
+      <c r="E411" t="str">
+        <v>Unison Group Com</v>
+      </c>
+      <c r="F411" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G411" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-unison-group-hyderabad-5-to-7-years-270126501900</v>
+      </c>
+      <c r="H411" t="str">
+        <v>https://apply.workable.com/unisongroup/j/C9D5349989</v>
+      </c>
+      <c r="I411" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412">
+        <v>411</v>
+      </c>
+      <c r="B412" t="str">
+        <v>27/5/2026, 11:39:18 am</v>
+      </c>
+      <c r="C412" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D412" t="str">
+        <v>Tech Lead - .Net Full Stack + Azure Integration Developer</v>
+      </c>
+      <c r="E412" t="str">
+        <v>Vlaunchu</v>
+      </c>
+      <c r="F412" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G412" t="str">
+        <v>https://www.naukri.com/job-listings-tech-lead-net-full-stack-azure-integration-developer-vlaunchu-hyderabad-6-to-8-years-261125501659</v>
+      </c>
+      <c r="H412" t="str">
+        <v>https://app.pyjamahr.com/careers?company=Vlaunchu&amp;job_id=275810&amp;company_uuid=DD8D585B0A</v>
+      </c>
+      <c r="I412" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413">
+        <v>412</v>
+      </c>
+      <c r="B413" t="str">
+        <v>27/5/2026, 11:39:23 am</v>
+      </c>
+      <c r="C413" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D413" t="str">
+        <v>Dot Net Full stack Developer</v>
+      </c>
+      <c r="E413" t="str">
+        <v>Stack Digital</v>
+      </c>
+      <c r="F413" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G413" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-stack-digital-warangal-hyderabad-nizamabad-6-to-11-years-260526506348</v>
+      </c>
+      <c r="H413" t="str">
+        <v>https://www.gostack.co.in/careers?job_id=z5G7h3l6a1kMvyS65NP3c5zEuNpzDuYog04XnU730ew=</v>
+      </c>
+      <c r="I413" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414">
+        <v>413</v>
+      </c>
+      <c r="B414" t="str">
+        <v>27/5/2026, 11:39:27 am</v>
+      </c>
+      <c r="C414" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D414" t="str">
+        <v>LBG -Full Stack Developer- Core Java</v>
+      </c>
+      <c r="E414" t="str">
+        <v>Krazymantra It Solutions</v>
+      </c>
+      <c r="F414" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G414" t="str">
+        <v>https://www.naukri.com/job-listings-lbg-full-stack-developer-core-java-krazymantra-it-solutions-hyderabad-bengaluru-10-to-15-years-260526505390</v>
+      </c>
+      <c r="H414" t="str">
+        <v>https://www.kmhr.in/job_description.php?id=1460</v>
+      </c>
+      <c r="I414" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415">
+        <v>414</v>
+      </c>
+      <c r="B415" t="str">
+        <v>27/5/2026, 11:40:35 am</v>
+      </c>
+      <c r="C415" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D415" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E415" t="str">
+        <v>Grid Dynamics</v>
+      </c>
+      <c r="F415" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G415" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-grid-dynamics-hyderabad-3-to-8-years-010825506485</v>
+      </c>
+      <c r="H415" t="str">
+        <v>https://www.griddynamics.com/careers/discover-openings</v>
+      </c>
+      <c r="I415" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416">
+        <v>415</v>
+      </c>
+      <c r="B416" t="str">
+        <v>27/5/2026, 11:41:10 am</v>
+      </c>
+      <c r="C416" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D416" t="str">
+        <v>Dot NET Full Stack developer</v>
+      </c>
+      <c r="E416" t="str">
+        <v>Ztek Consulting</v>
+      </c>
+      <c r="F416" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G416" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-ztek-consulting-pvt-ltd-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-4-to-10-years-240625503738</v>
+      </c>
+      <c r="H416" t="str">
+        <v>https://futransolutions.com/careers/?job_id=z5G7h3l6a1kMvyS65NP3c-Br5hzrhwV6T90VxvIu_kk=</v>
+      </c>
+      <c r="I416" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417">
+        <v>416</v>
+      </c>
+      <c r="B417" t="str">
+        <v>27/5/2026, 11:41:54 am</v>
+      </c>
+      <c r="C417" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D417" t="str">
+        <v>Software Developer (Full Stack Developer)</v>
+      </c>
+      <c r="E417" t="str">
+        <v>Qualcomm</v>
+      </c>
+      <c r="F417" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G417" t="str">
+        <v>https://www.naukri.com/job-listings-software-developer-full-stack-developer-qualcomm-india-pvt-ltd-hyderabad-3-to-5-years-250526912493</v>
+      </c>
+      <c r="H417" t="str">
+        <v>https://careers.qualcomm.com/careers?pid=446718579136</v>
+      </c>
+      <c r="I417" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418">
+        <v>417</v>
+      </c>
+      <c r="B418" t="str">
+        <v>27/5/2026, 11:45:04 am</v>
+      </c>
+      <c r="C418" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D418" t="str">
+        <v>Junior Full Stack Developer ( ColdFusion )</v>
+      </c>
+      <c r="E418" t="str">
+        <v>Infoane</v>
+      </c>
+      <c r="F418" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G418" t="str">
+        <v>https://www.naukri.com/job-listings-junior-full-stack-developer-coldfusion-infoane-technologies-hyderabad-0-to-2-years-270625503090</v>
+      </c>
+      <c r="H418" t="str">
+        <v>https://www.infoanetech.com/career.html</v>
+      </c>
+      <c r="I418" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419">
+        <v>418</v>
+      </c>
+      <c r="B419" t="str">
+        <v>27/5/2026, 11:45:24 am</v>
+      </c>
+      <c r="C419" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D419" t="str">
+        <v>Dotnet Full Stack Developer</v>
+      </c>
+      <c r="E419" t="str">
+        <v>Covalense Global</v>
+      </c>
+      <c r="F419" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G419" t="str">
+        <v>https://www.naukri.com/job-listings-dotnet-full-stack-developer-covalense-global-hyderabad-10-to-15-years-210526504311</v>
+      </c>
+      <c r="H419" t="str">
+        <v>https://www.covalenseglobal.com/jobs/net-full-stack-developer</v>
+      </c>
+      <c r="I419" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420">
+        <v>419</v>
+      </c>
+      <c r="B420" t="str">
+        <v>27/5/2026, 11:45:30 am</v>
+      </c>
+      <c r="C420" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D420" t="str">
+        <v>Dot Net Full Stack Developer</v>
+      </c>
+      <c r="E420" t="str">
+        <v>CloudStakes</v>
+      </c>
+      <c r="F420" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G420" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-cloudstakes-technology-pvt-ltd-hyderabad-8-to-12-years-210526500034</v>
+      </c>
+      <c r="H420" t="str">
+        <v>https://cloudstakes.com/careers</v>
+      </c>
+      <c r="I420" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421">
+        <v>420</v>
+      </c>
+      <c r="B421" t="str">
+        <v>27/5/2026, 11:46:15 am</v>
+      </c>
+      <c r="C421" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D421" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E421" t="str">
+        <v>TAO Digital</v>
+      </c>
+      <c r="F421" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G421" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-tao-digital-india-private-limited-hyderabad-8-to-13-years-260325503979</v>
+      </c>
+      <c r="H421" t="str">
+        <v>https://www.taodigitalsolutions.com/careers?job_id=z5G7h3l6a1kMvyS65NP3c0bHoot6yCaVHFzau4samhM=</v>
+      </c>
+      <c r="I421" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422">
+        <v>421</v>
+      </c>
+      <c r="B422" t="str">
+        <v>27/5/2026, 11:47:46 am</v>
+      </c>
+      <c r="C422" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D422" t="str">
+        <v>Lead Dot net full stack developer</v>
+      </c>
+      <c r="E422" t="str">
+        <v>Tech Stalwart Solution</v>
+      </c>
+      <c r="F422" t="str">
+        <v>Hyderabad, Mumbai, Kolkata, New Delhi, Pune, Chennai, Bengaluru</v>
+      </c>
+      <c r="G422" t="str">
+        <v>https://www.naukri.com/job-listings-lead-dot-net-full-stack-developer-tech-stalwart-solution-private-limited-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-10-years-100625502525</v>
+      </c>
+      <c r="H422" t="str">
+        <v>https://techstalwartsolution.com/career.html?job_id=z5G7h3l6a1kMvyS65NP3cxw5UCkv8X9vuzGaio8K7ys=</v>
+      </c>
+      <c r="I422" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423">
+        <v>422</v>
+      </c>
+      <c r="B423" t="str">
+        <v>27/5/2026, 11:47:58 am</v>
+      </c>
+      <c r="C423" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D423" t="str">
+        <v>Dot Net Full Stack Developer</v>
+      </c>
+      <c r="E423" t="str">
+        <v>Criticalriver</v>
+      </c>
+      <c r="F423" t="str">
+        <v>Hyderabad, Warangal, Nizamabad</v>
+      </c>
+      <c r="G423" t="str">
+        <v>https://www.naukri.com/job-listings-dot-net-full-stack-developer-criticalriver-inc-warangal-hyderabad-nizamabad-2-to-7-years-281125500686</v>
+      </c>
+      <c r="H423" t="str">
+        <v>https://www.criticalriver.com/apac-india-jobs/?job_id=z5G7h3l6a1kMvyS65NP3c13b6cpGhaN_qQCmBwMZqJw=</v>
+      </c>
+      <c r="I423" t="str">
+        <v>External — apply manually</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I388"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I423"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -14212,7 +15430,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I275"/>
+  <dimension ref="A1:I338"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -22200,9 +23418,1836 @@
         <v>chatbot_unknown</v>
       </c>
     </row>
+    <row r="276">
+      <c r="A276">
+        <v>275</v>
+      </c>
+      <c r="B276" t="str">
+        <v>27/5/2026, 11:33:36 am</v>
+      </c>
+      <c r="C276" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D276" t="str">
+        <v>Java Full Stack Developer/ Mern full stack developer (2 years+)</v>
+      </c>
+      <c r="E276" t="str">
+        <v>Premier Solar Systems</v>
+      </c>
+      <c r="F276" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G276" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-mern-full-stack-developer-2-years-premier-solar-systems-hyderabad-2-to-3-years-220526025780</v>
+      </c>
+      <c r="H276" t="str">
+        <v/>
+      </c>
+      <c r="I276" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277">
+        <v>276</v>
+      </c>
+      <c r="B277" t="str">
+        <v>27/5/2026, 11:34:29 am</v>
+      </c>
+      <c r="C277" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D277" t="str">
+        <v>Senior Developer (Full Stack)</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Nxtwave Disruptive Technologies (Hiring for a client)</v>
+      </c>
+      <c r="F277" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G277" t="str">
+        <v>https://www.naukri.com/job-listings-senior-developer-full-stack-nxtwave-disruptive-technologies-hiring-for-a-client-hyderabad-2-to-5-years-260526038661</v>
+      </c>
+      <c r="H277" t="str">
+        <v/>
+      </c>
+      <c r="I277" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278">
+        <v>277</v>
+      </c>
+      <c r="B278" t="str">
+        <v>27/5/2026, 11:35:01 am</v>
+      </c>
+      <c r="C278" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Full Stack .Net Developer</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Advintek</v>
+      </c>
+      <c r="F278" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G278" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-net-developer-advintek-hyderabad-2-to-5-years-230226012177</v>
+      </c>
+      <c r="H278" t="str">
+        <v/>
+      </c>
+      <c r="I278" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279">
+        <v>278</v>
+      </c>
+      <c r="B279" t="str">
+        <v>27/5/2026, 11:35:23 am</v>
+      </c>
+      <c r="C279" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Soc Software</v>
+      </c>
+      <c r="F279" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G279" t="str">
+        <v>https://www.naukri.com/job-listings-software-engineer-soc-software-hyderabad-1-to-3-years-260526027418</v>
+      </c>
+      <c r="H279" t="str">
+        <v/>
+      </c>
+      <c r="I279" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280">
+        <v>279</v>
+      </c>
+      <c r="B280" t="str">
+        <v>27/5/2026, 11:35:42 am</v>
+      </c>
+      <c r="C280" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D280" t="str">
+        <v>Full stack developer</v>
+      </c>
+      <c r="E280" t="str">
+        <v>Cognizant</v>
+      </c>
+      <c r="F280" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G280" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-cognizant-hyderabad-6-to-7-years-200526037003</v>
+      </c>
+      <c r="H280" t="str">
+        <v/>
+      </c>
+      <c r="I280" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" t="str">
+        <v>27/5/2026, 11:36:04 am</v>
+      </c>
+      <c r="C281" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Walk-in || Azure +.Net Full Stack Developer</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F281" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G281" t="str">
+        <v>https://www.naukri.com/job-listings-azure-net-full-stack-developer-tata-consultancy-services-hyderabad-6-to-10-years-260526012706</v>
+      </c>
+      <c r="H281" t="str">
+        <v/>
+      </c>
+      <c r="I281" t="str">
+        <v>no_apply_button</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282">
+        <v>281</v>
+      </c>
+      <c r="B282" t="str">
+        <v>27/5/2026, 11:36:12 am</v>
+      </c>
+      <c r="C282" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D282" t="str">
+        <v>Full Stack Developer</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Victrix Systems And Labs</v>
+      </c>
+      <c r="F282" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G282" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-victrix-systems-and-labs-hyderabad-6-to-8-years-200526916169</v>
+      </c>
+      <c r="H282" t="str">
+        <v/>
+      </c>
+      <c r="I282" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283">
+        <v>282</v>
+      </c>
+      <c r="B283" t="str">
+        <v>27/5/2026, 11:36:26 am</v>
+      </c>
+      <c r="C283" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Full Stack Developer-AI</v>
+      </c>
+      <c r="E283" t="str">
+        <v>INTERNAL</v>
+      </c>
+      <c r="F283" t="str">
+        <v>Hybrid - Hyderabad, Gurugram, Bengaluru</v>
+      </c>
+      <c r="G283" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-ai-joulestowatts-hyderabad-gurugram-bengaluru-7-to-12-years-200526012417</v>
+      </c>
+      <c r="H283" t="str">
+        <v/>
+      </c>
+      <c r="I283" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" t="str">
+        <v>27/5/2026, 11:36:34 am</v>
+      </c>
+      <c r="C284" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D284" t="str">
+        <v>AWS Full stack developer</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Coforge</v>
+      </c>
+      <c r="F284" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G284" t="str">
+        <v>https://www.naukri.com/job-listings-aws-full-stack-developer-coforge-hyderabad-pune-bengaluru-6-to-11-years-190526038688</v>
+      </c>
+      <c r="H284" t="str">
+        <v/>
+      </c>
+      <c r="I284" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285">
+        <v>284</v>
+      </c>
+      <c r="B285" t="str">
+        <v>27/5/2026, 11:36:50 am</v>
+      </c>
+      <c r="C285" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D285" t="str">
+        <v>GenAI Full Stack Developer</v>
+      </c>
+      <c r="E285" t="str">
+        <v>PwC Service Delivery Center</v>
+      </c>
+      <c r="F285" t="str">
+        <v>Hybrid - Hyderabad, Kolkata, Bengaluru</v>
+      </c>
+      <c r="G285" t="str">
+        <v>https://www.naukri.com/job-listings-genai-full-stack-developer-pwc-service-delivery-center-kolkata-hyderabad-bengaluru-4-to-8-years-210526027379</v>
+      </c>
+      <c r="H285" t="str">
+        <v/>
+      </c>
+      <c r="I285" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286">
+        <v>285</v>
+      </c>
+      <c r="B286" t="str">
+        <v>27/5/2026, 11:37:38 am</v>
+      </c>
+      <c r="C286" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D286" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E286" t="str">
+        <v>Yash Technologies</v>
+      </c>
+      <c r="F286" t="str">
+        <v>Hyderabad, Indore, Pune</v>
+      </c>
+      <c r="G286" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-yash-technologies-indore-hyderabad-pune-5-to-9-years-270426003813</v>
+      </c>
+      <c r="H286" t="str">
+        <v/>
+      </c>
+      <c r="I286" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287">
+        <v>286</v>
+      </c>
+      <c r="B287" t="str">
+        <v>27/5/2026, 11:37:46 am</v>
+      </c>
+      <c r="C287" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D287" t="str">
+        <v>Hiring For .NET Full stack React JS Developer</v>
+      </c>
+      <c r="E287" t="str">
+        <v>Tech Mahindra</v>
+      </c>
+      <c r="F287" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G287" t="str">
+        <v>https://www.naukri.com/job-listings-hiring-for-net-full-stack-react-js-developer-tech-mahindra-hyderabad-chennai-bengaluru-6-to-10-years-270426003698</v>
+      </c>
+      <c r="H287" t="str">
+        <v/>
+      </c>
+      <c r="I287" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288">
+        <v>287</v>
+      </c>
+      <c r="B288" t="str">
+        <v>27/5/2026, 11:38:13 am</v>
+      </c>
+      <c r="C288" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D288" t="str">
+        <v>Java Full Stack Developer with React Js</v>
+      </c>
+      <c r="E288" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F288" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G288" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-with-react-js-tata-consultancy-services-hyderabad-chennai-bengaluru-5-to-10-years-270426001953</v>
+      </c>
+      <c r="H288" t="str">
+        <v/>
+      </c>
+      <c r="I288" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289">
+        <v>288</v>
+      </c>
+      <c r="B289" t="str">
+        <v>27/5/2026, 11:38:21 am</v>
+      </c>
+      <c r="C289" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F289" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G289" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-11-years-270426001711</v>
+      </c>
+      <c r="H289" t="str">
+        <v/>
+      </c>
+      <c r="I289" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290">
+        <v>289</v>
+      </c>
+      <c r="B290" t="str">
+        <v>27/5/2026, 11:39:54 am</v>
+      </c>
+      <c r="C290" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E290" t="str">
+        <v>Randomtrees</v>
+      </c>
+      <c r="F290" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G290" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-randomtrees-hyderabad-7-to-10-years-260526038695</v>
+      </c>
+      <c r="H290" t="str">
+        <v/>
+      </c>
+      <c r="I290" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291">
+        <v>290</v>
+      </c>
+      <c r="B291" t="str">
+        <v>27/5/2026, 11:40:02 am</v>
+      </c>
+      <c r="C291" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E291" t="str">
+        <v>Trackmind Solutions</v>
+      </c>
+      <c r="F291" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G291" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-trackmind-solutions-hyderabad-3-to-5-years-250526009924</v>
+      </c>
+      <c r="H291" t="str">
+        <v/>
+      </c>
+      <c r="I291" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292">
+        <v>291</v>
+      </c>
+      <c r="B292" t="str">
+        <v>27/5/2026, 11:40:29 am</v>
+      </c>
+      <c r="C292" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D292" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E292" t="str">
+        <v>Trackmind Solutions</v>
+      </c>
+      <c r="F292" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G292" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-trackmind-solutions-hyderabad-3-to-7-years-250526009129</v>
+      </c>
+      <c r="H292" t="str">
+        <v/>
+      </c>
+      <c r="I292" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293">
+        <v>292</v>
+      </c>
+      <c r="B293" t="str">
+        <v>27/5/2026, 11:41:02 am</v>
+      </c>
+      <c r="C293" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Java Full Stack Developer (Angular/Reactjs) hyd</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F293" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G293" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-angular-reactjs-hyd-infosys-hyderabad-3-to-8-years-250526003614</v>
+      </c>
+      <c r="H293" t="str">
+        <v/>
+      </c>
+      <c r="I293" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294">
+        <v>293</v>
+      </c>
+      <c r="B294" t="str">
+        <v>27/5/2026, 11:41:18 am</v>
+      </c>
+      <c r="C294" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Fullstack AI Developer</v>
+      </c>
+      <c r="E294" t="str">
+        <v>Intellisavvy</v>
+      </c>
+      <c r="F294" t="str">
+        <v>Hyderabad(Madhapur), Visakhapatnam(Siripuram)</v>
+      </c>
+      <c r="G294" t="str">
+        <v>https://www.naukri.com/job-listings-fullstack-ai-developer-intellisavvy-visakhapatnam-hyderabad-4-to-7-years-210526027902</v>
+      </c>
+      <c r="H294" t="str">
+        <v/>
+      </c>
+      <c r="I294" t="str">
+        <v>chatbot_unknown</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295">
+        <v>294</v>
+      </c>
+      <c r="B295" t="str">
+        <v>27/5/2026, 11:41:25 am</v>
+      </c>
+      <c r="C295" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D295" t="str">
+        <v>Virtusa actively looking For Full Stack Developers</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Virtusa</v>
+      </c>
+      <c r="F295" t="str">
+        <v>Hyderabad, Chennai</v>
+      </c>
+      <c r="G295" t="str">
+        <v>https://www.naukri.com/job-listings-virtusa-actively-looking-for-full-stack-developers-virtusa-hyderabad-chennai-5-to-9-years-220526028549</v>
+      </c>
+      <c r="H295" t="str">
+        <v/>
+      </c>
+      <c r="I295" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296">
+        <v>295</v>
+      </c>
+      <c r="B296" t="str">
+        <v>27/5/2026, 11:42:02 am</v>
+      </c>
+      <c r="C296" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Azure .NET Full Stack Developer</v>
+      </c>
+      <c r="E296" t="str">
+        <v>ti Steps</v>
+      </c>
+      <c r="F296" t="str">
+        <v>Hyderabad, Bengaluru</v>
+      </c>
+      <c r="G296" t="str">
+        <v>https://www.naukri.com/job-listings-azure-net-full-stack-developer-ti-steps-hyderabad-bengaluru-5-to-8-years-260526016897</v>
+      </c>
+      <c r="H296" t="str">
+        <v/>
+      </c>
+      <c r="I296" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297">
+        <v>296</v>
+      </c>
+      <c r="B297" t="str">
+        <v>27/5/2026, 11:42:10 am</v>
+      </c>
+      <c r="C297" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D297" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E297" t="str">
+        <v>with one of our Level 5 Client</v>
+      </c>
+      <c r="F297" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G297" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-bcforward-hyderabad-6-to-11-years-250526920310</v>
+      </c>
+      <c r="H297" t="str">
+        <v/>
+      </c>
+      <c r="I297" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298">
+        <v>297</v>
+      </c>
+      <c r="B298" t="str">
+        <v>27/5/2026, 11:42:18 am</v>
+      </c>
+      <c r="C298" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D298" t="str">
+        <v>.NET Core full stack developer</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F298" t="str">
+        <v>Hybrid - Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G298" t="str">
+        <v>https://www.naukri.com/job-listings-net-core-full-stack-developer-infosys-hyderabad-chennai-bengaluru-3-to-8-years-220526031957</v>
+      </c>
+      <c r="H298" t="str">
+        <v/>
+      </c>
+      <c r="I298" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299">
+        <v>298</v>
+      </c>
+      <c r="B299" t="str">
+        <v>27/5/2026, 11:42:26 am</v>
+      </c>
+      <c r="C299" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Full Stack Developer - .Net</v>
+      </c>
+      <c r="E299" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F299" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G299" t="str">
+        <v>https://www.naukri.com/job-listings-full-stack-developer-net-4s-advisory-hyderabad-8-to-10-years-210526922437</v>
+      </c>
+      <c r="H299" t="str">
+        <v/>
+      </c>
+      <c r="I299" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300">
+        <v>299</v>
+      </c>
+      <c r="B300" t="str">
+        <v>27/5/2026, 11:42:34 am</v>
+      </c>
+      <c r="C300" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Sr Java with Vue.js Full Stack Developer</v>
+      </c>
+      <c r="E300" t="str">
+        <v>Deloitte US-India Offices</v>
+      </c>
+      <c r="F300" t="str">
+        <v>Hyderabad, Bengaluru, Delhi / NCR</v>
+      </c>
+      <c r="G300" t="str">
+        <v>https://www.naukri.com/job-listings-sr-java-with-vue-js-full-stack-developer-deloitte-us-india-offices-hyderabad-bengaluru-delhi-ncr-7-to-12-years-260526018258</v>
+      </c>
+      <c r="H300" t="str">
+        <v/>
+      </c>
+      <c r="I300" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301">
+        <v>300</v>
+      </c>
+      <c r="B301" t="str">
+        <v>27/5/2026, 11:42:53 am</v>
+      </c>
+      <c r="C301" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F301" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G301" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-4-to-8-years-200426007243</v>
+      </c>
+      <c r="H301" t="str">
+        <v/>
+      </c>
+      <c r="I301" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" t="str">
+        <v>27/5/2026, 11:43:01 am</v>
+      </c>
+      <c r="C302" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Java Full stack developer</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F302" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G302" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-infosys-limited-hyderabad-3-to-8-years-210526923113</v>
+      </c>
+      <c r="H302" t="str">
+        <v/>
+      </c>
+      <c r="I302" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303">
+        <v>302</v>
+      </c>
+      <c r="B303" t="str">
+        <v>27/5/2026, 11:43:09 am</v>
+      </c>
+      <c r="C303" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Careernet</v>
+      </c>
+      <c r="F303" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G303" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-careernet-hyderabad-5-to-8-years-250326027915</v>
+      </c>
+      <c r="H303" t="str">
+        <v/>
+      </c>
+      <c r="I303" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304">
+        <v>303</v>
+      </c>
+      <c r="B304" t="str">
+        <v>27/5/2026, 11:43:16 am</v>
+      </c>
+      <c r="C304" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Senior Java Full Stack Developer</v>
+      </c>
+      <c r="E304" t="str">
+        <v>CGI</v>
+      </c>
+      <c r="F304" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G304" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-cgi-information-systems-and-management-consultants-hyderabad-5-to-10-years-210526923117</v>
+      </c>
+      <c r="H304" t="str">
+        <v/>
+      </c>
+      <c r="I304" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305">
+        <v>304</v>
+      </c>
+      <c r="B305" t="str">
+        <v>27/5/2026, 11:43:24 am</v>
+      </c>
+      <c r="C305" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Vue JS Full-Stack Developer</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F305" t="str">
+        <v>Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G305" t="str">
+        <v>https://www.naukri.com/job-listings-vue-js-full-stack-developer-tata-consultancy-services-hyderabad-pune-bengaluru-5-to-10-years-210526015289</v>
+      </c>
+      <c r="H305" t="str">
+        <v/>
+      </c>
+      <c r="I305" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306">
+        <v>305</v>
+      </c>
+      <c r="B306" t="str">
+        <v>27/5/2026, 11:43:32 am</v>
+      </c>
+      <c r="C306" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G306" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-9-years-210526014531</v>
+      </c>
+      <c r="H306" t="str">
+        <v/>
+      </c>
+      <c r="I306" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307">
+        <v>306</v>
+      </c>
+      <c r="B307" t="str">
+        <v>27/5/2026, 11:43:40 am</v>
+      </c>
+      <c r="C307" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Java Full stack Developer with Angular/React</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Crisil</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G307" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-with-angular-react-crisil-hyderabad-8-to-12-years-210526013696</v>
+      </c>
+      <c r="H307" t="str">
+        <v/>
+      </c>
+      <c r="I307" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308">
+        <v>307</v>
+      </c>
+      <c r="B308" t="str">
+        <v>27/5/2026, 11:43:48 am</v>
+      </c>
+      <c r="C308" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Senior Full-Stack Developer (Immediate Joiners Only)</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Straive</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G308" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-immediate-joiners-only-straive-hyderabad-pune-bengaluru-5-to-6-years-200526030228</v>
+      </c>
+      <c r="H308" t="str">
+        <v/>
+      </c>
+      <c r="I308" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309">
+        <v>308</v>
+      </c>
+      <c r="B309" t="str">
+        <v>27/5/2026, 11:43:56 am</v>
+      </c>
+      <c r="C309" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Trackmind Solutions</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G309" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-trackmind-solutions-hyderabad-3-to-6-years-250526009745</v>
+      </c>
+      <c r="H309" t="str">
+        <v/>
+      </c>
+      <c r="I309" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310">
+        <v>309</v>
+      </c>
+      <c r="B310" t="str">
+        <v>27/5/2026, 11:44:04 am</v>
+      </c>
+      <c r="C310" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Tredence</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G310" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-tredence-hyderabad-pune-bengaluru-5-to-8-years-260526036576</v>
+      </c>
+      <c r="H310" t="str">
+        <v/>
+      </c>
+      <c r="I310" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311">
+        <v>310</v>
+      </c>
+      <c r="B311" t="str">
+        <v>27/5/2026, 11:44:12 am</v>
+      </c>
+      <c r="C311" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D311" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E311" t="str">
+        <v>People Prime Worldwide</v>
+      </c>
+      <c r="F311" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G311" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-people-prime-worldwide-hyderabad-6-to-8-years-260526025410</v>
+      </c>
+      <c r="H311" t="str">
+        <v/>
+      </c>
+      <c r="I311" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312">
+        <v>311</v>
+      </c>
+      <c r="B312" t="str">
+        <v>27/5/2026, 11:44:20 am</v>
+      </c>
+      <c r="C312" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Angular Full Stack Developer</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G312" t="str">
+        <v>https://www.naukri.com/job-listings-angular-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-5-to-10-years-260526022671</v>
+      </c>
+      <c r="H312" t="str">
+        <v/>
+      </c>
+      <c r="I312" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313">
+        <v>312</v>
+      </c>
+      <c r="B313" t="str">
+        <v>27/5/2026, 11:44:28 am</v>
+      </c>
+      <c r="C313" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Senior .NET Full-stack Developer</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Cirruslabs</v>
+      </c>
+      <c r="F313" t="str">
+        <v>Hybrid - Hyderabad, Mangaluru, Bengaluru</v>
+      </c>
+      <c r="G313" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-cirruslabs-hyderabad-mangaluru-bengaluru-6-to-10-years-260526015566</v>
+      </c>
+      <c r="H313" t="str">
+        <v/>
+      </c>
+      <c r="I313" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314">
+        <v>313</v>
+      </c>
+      <c r="B314" t="str">
+        <v>27/5/2026, 11:44:35 am</v>
+      </c>
+      <c r="C314" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D314" t="str">
+        <v>.NET Full Stack Developer</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F314" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G314" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-bcforward-india-technologies-private-limited-hyderabad-10-to-15-years-250526924975</v>
+      </c>
+      <c r="H314" t="str">
+        <v/>
+      </c>
+      <c r="I314" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315">
+        <v>314</v>
+      </c>
+      <c r="B315" t="str">
+        <v>27/5/2026, 11:44:43 am</v>
+      </c>
+      <c r="C315" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D315" t="str">
+        <v>.Net Full Stack Developer- C2H Role</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G315" t="str">
+        <v>https://www.naukri.com/job-listings-net-full-stack-developer-c2h-role-bcforward-india-technologies-private-limited-hyderabad-5-to-10-years-250526921208</v>
+      </c>
+      <c r="H315" t="str">
+        <v/>
+      </c>
+      <c r="I315" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316">
+        <v>315</v>
+      </c>
+      <c r="B316" t="str">
+        <v>27/5/2026, 11:44:51 am</v>
+      </c>
+      <c r="C316" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E316" t="str">
+        <v>with one of our client</v>
+      </c>
+      <c r="F316" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G316" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-bcforward-hyderabad-10-to-15-years-250526919884</v>
+      </c>
+      <c r="H316" t="str">
+        <v/>
+      </c>
+      <c r="I316" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317">
+        <v>316</v>
+      </c>
+      <c r="B317" t="str">
+        <v>27/5/2026, 11:44:59 am</v>
+      </c>
+      <c r="C317" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D317" t="str">
+        <v>Java Full Stack developer(React JS)</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F317" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G317" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-react-js-infosys-hyderabad-pune-bengaluru-5-to-9-years-220526031884</v>
+      </c>
+      <c r="H317" t="str">
+        <v/>
+      </c>
+      <c r="I317" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318">
+        <v>317</v>
+      </c>
+      <c r="B318" t="str">
+        <v>27/5/2026, 11:45:12 am</v>
+      </c>
+      <c r="C318" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Senior Java Full Stack Developer</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Luxoft</v>
+      </c>
+      <c r="F318" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G318" t="str">
+        <v>https://www.naukri.com/job-listings-senior-java-full-stack-developer-luxoft-india-llp-hyderabad-6-to-10-years-220526929571</v>
+      </c>
+      <c r="H318" t="str">
+        <v/>
+      </c>
+      <c r="I318" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319">
+        <v>318</v>
+      </c>
+      <c r="B319" t="str">
+        <v>27/5/2026, 11:45:20 am</v>
+      </c>
+      <c r="C319" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Senior Full Stack Developer (iOS + React)</v>
+      </c>
+      <c r="E319" t="str">
+        <v>iSpatial Techno</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G319" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-ios-react-ispatial-techno-hyderabad-5-to-10-years-210526918733</v>
+      </c>
+      <c r="H319" t="str">
+        <v/>
+      </c>
+      <c r="I319" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320">
+        <v>319</v>
+      </c>
+      <c r="B320" t="str">
+        <v>27/5/2026, 11:45:38 am</v>
+      </c>
+      <c r="C320" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Vue JS Full-Stack Developer</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F320" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G320" t="str">
+        <v>https://www.naukri.com/job-listings-vue-js-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-5-to-10-years-210526016709</v>
+      </c>
+      <c r="H320" t="str">
+        <v/>
+      </c>
+      <c r="I320" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321">
+        <v>320</v>
+      </c>
+      <c r="B321" t="str">
+        <v>27/5/2026, 11:45:46 am</v>
+      </c>
+      <c r="C321" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Soothsayer Analytics</v>
+      </c>
+      <c r="F321" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G321" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-soothsayer-analytics-hyderabad-8-to-10-years-200526917318</v>
+      </c>
+      <c r="H321" t="str">
+        <v/>
+      </c>
+      <c r="I321" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322">
+        <v>321</v>
+      </c>
+      <c r="B322" t="str">
+        <v>27/5/2026, 11:45:54 am</v>
+      </c>
+      <c r="C322" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Senior Full Stack Developer</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Careernet</v>
+      </c>
+      <c r="F322" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G322" t="str">
+        <v>https://www.naukri.com/job-listings-senior-full-stack-developer-careernet-hyderabad-5-to-7-years-200526044560</v>
+      </c>
+      <c r="H322" t="str">
+        <v/>
+      </c>
+      <c r="I322" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323">
+        <v>322</v>
+      </c>
+      <c r="B323" t="str">
+        <v>27/5/2026, 11:46:02 am</v>
+      </c>
+      <c r="C323" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F323" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G323" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-10-years-200526030342</v>
+      </c>
+      <c r="H323" t="str">
+        <v/>
+      </c>
+      <c r="I323" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324">
+        <v>323</v>
+      </c>
+      <c r="B324" t="str">
+        <v>27/5/2026, 11:46:10 am</v>
+      </c>
+      <c r="C324" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Java Full Stack Developer/Lead</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Hexaware Technologies</v>
+      </c>
+      <c r="F324" t="str">
+        <v>Hybrid - Hyderabad, Pune, Chennai</v>
+      </c>
+      <c r="G324" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-lead-hexaware-technologies-hyderabad-pune-chennai-6-to-11-years-060526013998</v>
+      </c>
+      <c r="H324" t="str">
+        <v/>
+      </c>
+      <c r="I324" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325">
+        <v>324</v>
+      </c>
+      <c r="B325" t="str">
+        <v>27/5/2026, 11:46:23 am</v>
+      </c>
+      <c r="C325" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F325" t="str">
+        <v>Hyderabad, Kochi, Chennai</v>
+      </c>
+      <c r="G325" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-wipro-kochi-hyderabad-chennai-5-to-8-years-260526023906</v>
+      </c>
+      <c r="H325" t="str">
+        <v/>
+      </c>
+      <c r="I325" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326">
+        <v>325</v>
+      </c>
+      <c r="B326" t="str">
+        <v>27/5/2026, 11:46:31 am</v>
+      </c>
+      <c r="C326" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F326" t="str">
+        <v>Hyderabad, Pune, Chennai</v>
+      </c>
+      <c r="G326" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-pune-chennai-5-to-10-years-260526017381</v>
+      </c>
+      <c r="H326" t="str">
+        <v/>
+      </c>
+      <c r="I326" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327">
+        <v>326</v>
+      </c>
+      <c r="B327" t="str">
+        <v>27/5/2026, 11:46:39 am</v>
+      </c>
+      <c r="C327" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D327" t="str">
+        <v>react -java full stack developer</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Cloudxtreme</v>
+      </c>
+      <c r="F327" t="str">
+        <v>Hyderabad, Bengaluru, Delhi / NCR</v>
+      </c>
+      <c r="G327" t="str">
+        <v>https://www.naukri.com/job-listings-react-java-full-stack-developer-cloudxtreme-hyderabad-bengaluru-delhi-ncr-8-to-12-years-260326014840</v>
+      </c>
+      <c r="H327" t="str">
+        <v/>
+      </c>
+      <c r="I327" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328">
+        <v>327</v>
+      </c>
+      <c r="B328" t="str">
+        <v>27/5/2026, 11:46:47 am</v>
+      </c>
+      <c r="C328" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E328" t="str">
+        <v>IT Industry</v>
+      </c>
+      <c r="F328" t="str">
+        <v>Hyderabad, Bengaluru, Delhi / NCR</v>
+      </c>
+      <c r="G328" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-serendipity-corporate-services-hyderabad-bengaluru-delhi-ncr-5-to-9-years-250526926866</v>
+      </c>
+      <c r="H328" t="str">
+        <v/>
+      </c>
+      <c r="I328" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329">
+        <v>328</v>
+      </c>
+      <c r="B329" t="str">
+        <v>27/5/2026, 11:46:55 am</v>
+      </c>
+      <c r="C329" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Leading Client</v>
+      </c>
+      <c r="F329" t="str">
+        <v>Hybrid - Hyderabad</v>
+      </c>
+      <c r="G329" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-bcforward-india-technologies-private-limited-hyderabad-8-to-13-years-250526923984</v>
+      </c>
+      <c r="H329" t="str">
+        <v/>
+      </c>
+      <c r="I329" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330">
+        <v>329</v>
+      </c>
+      <c r="B330" t="str">
+        <v>27/5/2026, 11:47:02 am</v>
+      </c>
+      <c r="C330" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E330" t="str">
+        <v>BCForward</v>
+      </c>
+      <c r="F330" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="G330" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-bcforward-hyderabad-5-to-7-years-250526919709</v>
+      </c>
+      <c r="H330" t="str">
+        <v/>
+      </c>
+      <c r="I330" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331">
+        <v>330</v>
+      </c>
+      <c r="B331" t="str">
+        <v>27/5/2026, 11:47:10 am</v>
+      </c>
+      <c r="C331" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Java Full Stack Developer</v>
+      </c>
+      <c r="E331" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F331" t="str">
+        <v>Hyderabad, Chennai, Bengaluru</v>
+      </c>
+      <c r="G331" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-tata-consultancy-services-hyderabad-chennai-bengaluru-6-to-10-years-250526037119</v>
+      </c>
+      <c r="H331" t="str">
+        <v/>
+      </c>
+      <c r="I331" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332">
+        <v>331</v>
+      </c>
+      <c r="B332" t="str">
+        <v>27/5/2026, 11:47:18 am</v>
+      </c>
+      <c r="C332" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D332" t="str">
+        <v>Java Full Stack Developer - Angular</v>
+      </c>
+      <c r="E332" t="str">
+        <v>Tata Consultancy Services</v>
+      </c>
+      <c r="F332" t="str">
+        <v>Hyderabad, Kolkata, Chennai</v>
+      </c>
+      <c r="G332" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-angular-tata-consultancy-services-kolkata-hyderabad-chennai-6-to-8-years-250526035751</v>
+      </c>
+      <c r="H332" t="str">
+        <v/>
+      </c>
+      <c r="I332" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333">
+        <v>332</v>
+      </c>
+      <c r="B333" t="str">
+        <v>27/5/2026, 11:47:26 am</v>
+      </c>
+      <c r="C333" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Python React Full Stack Developer</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Ascendion Engineering</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G333" t="str">
+        <v>https://www.naukri.com/job-listings-python-react-full-stack-developer-ascendion-engineering-hyderabad-pune-bengaluru-5-to-10-years-250526013440</v>
+      </c>
+      <c r="H333" t="str">
+        <v/>
+      </c>
+      <c r="I333" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334">
+        <v>333</v>
+      </c>
+      <c r="B334" t="str">
+        <v>27/5/2026, 11:47:34 am</v>
+      </c>
+      <c r="C334" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Senior .NET Full Stack Developer (Angular 12+ ,JavaScript ,.NET)</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Cirruslabs</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G334" t="str">
+        <v>https://www.naukri.com/job-listings-senior-net-full-stack-developer-angular-12-javascript-net-cirruslabs-hyderabad-pune-bengaluru-7-to-12-years-250526006421</v>
+      </c>
+      <c r="H334" t="str">
+        <v/>
+      </c>
+      <c r="I334" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335">
+        <v>334</v>
+      </c>
+      <c r="B335" t="str">
+        <v>27/5/2026, 11:47:42 am</v>
+      </c>
+      <c r="C335" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Java Full Stack developer(Angular JS) - Bengaluru</v>
+      </c>
+      <c r="E335" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F335" t="str">
+        <v>Hybrid - Hyderabad, Pune, Bengaluru</v>
+      </c>
+      <c r="G335" t="str">
+        <v>https://www.naukri.com/job-listings-java-full-stack-developer-angular-js-bengaluru-infosys-hyderabad-pune-bengaluru-5-to-9-years-210526015812</v>
+      </c>
+      <c r="H335" t="str">
+        <v/>
+      </c>
+      <c r="I335" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336">
+        <v>335</v>
+      </c>
+      <c r="B336" t="str">
+        <v>27/5/2026, 11:48:05 am</v>
+      </c>
+      <c r="C336" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D336" t="str">
+        <v>PLSQL Developer</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Solix Technologies</v>
+      </c>
+      <c r="F336" t="str">
+        <v>Hyderabad(HITEC City +2)</v>
+      </c>
+      <c r="G336" t="str">
+        <v>https://www.naukri.com/job-listings-plsql-developer-solix-technologies-hyderabad-3-to-4-years-270526014424</v>
+      </c>
+      <c r="H336" t="str">
+        <v/>
+      </c>
+      <c r="I336" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337">
+        <v>336</v>
+      </c>
+      <c r="B337" t="str">
+        <v>27/5/2026, 11:48:13 am</v>
+      </c>
+      <c r="C337" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Postgresql Database Administrator</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Solix Technologies</v>
+      </c>
+      <c r="F337" t="str">
+        <v>Hyderabad(HITEC City +2)</v>
+      </c>
+      <c r="G337" t="str">
+        <v>https://www.naukri.com/job-listings-postgresql-database-administrator-solix-technologies-hyderabad-4-to-8-years-260526029477</v>
+      </c>
+      <c r="H337" t="str">
+        <v/>
+      </c>
+      <c r="I337" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338">
+        <v>337</v>
+      </c>
+      <c r="B338" t="str">
+        <v>27/5/2026, 11:48:21 am</v>
+      </c>
+      <c r="C338" t="str">
+        <v>naukri</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Data Architect - SQL Server</v>
+      </c>
+      <c r="E338" t="str">
+        <v>Processq India</v>
+      </c>
+      <c r="F338" t="str">
+        <v>Hyderabad(HITEC City)</v>
+      </c>
+      <c r="G338" t="str">
+        <v>https://www.naukri.com/job-listings-data-architect-sql-server-processq-india-hyderabad-15-to-24-years-250526014629</v>
+      </c>
+      <c r="H338" t="str">
+        <v/>
+      </c>
+      <c r="I338" t="str">
+        <v>unknown_state</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I275"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I338"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>